<commit_message>
skill v2p9(config file provide input files) and rtm(plan mode)
</commit_message>
<xml_diff>
--- a/RTM_AI_FLTP_new.xlsx
+++ b/RTM_AI_FLTP_new.xlsx
@@ -1533,7 +1533,7 @@
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>CHK_002</t>
+          <t>CHK_001</t>
         </is>
       </c>
       <c r="F3" s="12" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>CHK_002</t>
+          <t>CHK_001</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="E5" s="18" t="inlineStr">
         <is>
-          <t>CHK_001</t>
+          <t>CHK_002</t>
         </is>
       </c>
       <c r="F5" s="18" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="E6" s="18" t="inlineStr">
         <is>
-          <t>CHK_001</t>
+          <t>CHK_002</t>
         </is>
       </c>
       <c r="F6" s="18" t="inlineStr">
@@ -1669,12 +1669,12 @@
       </c>
       <c r="E7" s="18" t="inlineStr">
         <is>
-          <t>CHK_003</t>
+          <t>CHK_003,CHK_004</t>
         </is>
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>TC_004,TC_050</t>
+          <t>TC_004,TC_055</t>
         </is>
       </c>
     </row>
@@ -1703,12 +1703,12 @@
       </c>
       <c r="E8" s="18" t="inlineStr">
         <is>
-          <t>CHK_003</t>
+          <t>CHK_004</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>TC_005,TC_034</t>
+          <t>TC_005</t>
         </is>
       </c>
     </row>
@@ -1737,12 +1737,12 @@
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>CHK_003</t>
+          <t>CHK_004</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>TC_006,TC_034</t>
+          <t>TC_006</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>CHK_004</t>
+          <t>CHK_005</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
@@ -1805,12 +1805,12 @@
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>CHK_004</t>
+          <t>CHK_005</t>
         </is>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>TC_007</t>
+          <t>TC_008</t>
         </is>
       </c>
     </row>
@@ -1839,12 +1839,12 @@
       </c>
       <c r="E12" s="18" t="inlineStr">
         <is>
-          <t>CHK_005</t>
+          <t>CHK_006</t>
         </is>
       </c>
       <c r="F12" s="18" t="inlineStr">
         <is>
-          <t>TC_008</t>
+          <t>TC_010</t>
         </is>
       </c>
     </row>
@@ -1873,12 +1873,12 @@
       </c>
       <c r="E13" s="18" t="inlineStr">
         <is>
-          <t>CHK_005</t>
+          <t>CHK_006</t>
         </is>
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
-          <t>TC_009</t>
+          <t>TC_011</t>
         </is>
       </c>
     </row>
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>CHK_005</t>
+          <t>CHK_006</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>TC_010</t>
+          <t>TC_012</t>
         </is>
       </c>
     </row>
@@ -1941,12 +1941,12 @@
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>CHK_005</t>
+          <t>CHK_006</t>
         </is>
       </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
-          <t>TC_011</t>
+          <t>TC_013</t>
         </is>
       </c>
     </row>
@@ -1975,12 +1975,12 @@
       </c>
       <c r="E16" s="18" t="inlineStr">
         <is>
-          <t>CHK_006</t>
+          <t>CHK_007</t>
         </is>
       </c>
       <c r="F16" s="18" t="inlineStr">
         <is>
-          <t>TC_012</t>
+          <t>TC_014</t>
         </is>
       </c>
     </row>
@@ -2009,12 +2009,12 @@
       </c>
       <c r="E17" s="18" t="inlineStr">
         <is>
-          <t>CHK_006</t>
+          <t>CHK_007</t>
         </is>
       </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
-          <t>TC_013</t>
+          <t>TC_015</t>
         </is>
       </c>
     </row>
@@ -2048,7 +2048,7 @@
       </c>
       <c r="F18" s="18" t="inlineStr">
         <is>
-          <t>TC_014</t>
+          <t>TC_016</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
-          <t>TC_015</t>
+          <t>TC_017</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>TC_016</t>
+          <t>TC_018</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
-          <t>TC_017</t>
+          <t>TC_019</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>TC_018</t>
+          <t>TC_020</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>TC_019</t>
+          <t>TC_021</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>TC_020</t>
+          <t>TC_022</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="F25" s="18" t="inlineStr">
         <is>
-          <t>TC_021</t>
+          <t>TC_023</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="F26" s="18" t="inlineStr">
         <is>
-          <t>TC_022</t>
+          <t>TC_024</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2354,7 @@
       </c>
       <c r="F27" s="18" t="inlineStr">
         <is>
-          <t>TC_023</t>
+          <t>TC_025</t>
         </is>
       </c>
     </row>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="F28" s="18" t="inlineStr">
         <is>
-          <t>TC_024</t>
+          <t>TC_026</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="F29" s="18" t="inlineStr">
         <is>
-          <t>TC_007,TC_051</t>
+          <t>TC_027</t>
         </is>
       </c>
     </row>
@@ -2451,12 +2451,12 @@
       </c>
       <c r="E30" s="18" t="inlineStr">
         <is>
-          <t>CHK_012</t>
+          <t>CHK_013</t>
         </is>
       </c>
       <c r="F30" s="18" t="inlineStr">
         <is>
-          <t>TC_039</t>
+          <t>TC_028</t>
         </is>
       </c>
     </row>
@@ -2485,12 +2485,12 @@
       </c>
       <c r="E31" s="18" t="inlineStr">
         <is>
-          <t>CHK_012</t>
+          <t>CHK_014</t>
         </is>
       </c>
       <c r="F31" s="18" t="inlineStr">
         <is>
-          <t>TC_025,TC_040</t>
+          <t>TC_029</t>
         </is>
       </c>
     </row>
@@ -2519,12 +2519,12 @@
       </c>
       <c r="E32" s="18" t="inlineStr">
         <is>
-          <t>CHK_012</t>
+          <t>CHK_015</t>
         </is>
       </c>
       <c r="F32" s="18" t="inlineStr">
         <is>
-          <t>TC_048</t>
+          <t>TC_030</t>
         </is>
       </c>
     </row>
@@ -2553,12 +2553,12 @@
       </c>
       <c r="E33" s="18" t="inlineStr">
         <is>
-          <t>CHK_012</t>
+          <t>CHK_015</t>
         </is>
       </c>
       <c r="F33" s="18" t="inlineStr">
         <is>
-          <t>TC_026,TC_041</t>
+          <t>TC_031</t>
         </is>
       </c>
     </row>
@@ -2587,12 +2587,12 @@
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>CHK_013</t>
+          <t>CHK_016</t>
         </is>
       </c>
       <c r="F34" s="18" t="inlineStr">
         <is>
-          <t>TC_035</t>
+          <t>TC_032</t>
         </is>
       </c>
     </row>
@@ -2621,12 +2621,12 @@
       </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
-          <t>CHK_013</t>
+          <t>CHK_016</t>
         </is>
       </c>
       <c r="F35" s="18" t="inlineStr">
         <is>
-          <t>TC_044</t>
+          <t>TC_033</t>
         </is>
       </c>
     </row>
@@ -2655,12 +2655,12 @@
       </c>
       <c r="E36" s="18" t="inlineStr">
         <is>
-          <t>CHK_013</t>
+          <t>CHK_017</t>
         </is>
       </c>
       <c r="F36" s="18" t="inlineStr">
         <is>
-          <t>TC_038</t>
+          <t>TC_034</t>
         </is>
       </c>
     </row>
@@ -2689,12 +2689,12 @@
       </c>
       <c r="E37" s="18" t="inlineStr">
         <is>
-          <t>CHK_014</t>
+          <t>CHK_018</t>
         </is>
       </c>
       <c r="F37" s="18" t="inlineStr">
         <is>
-          <t>TC_027</t>
+          <t>TC_035</t>
         </is>
       </c>
     </row>
@@ -2723,12 +2723,12 @@
       </c>
       <c r="E38" s="18" t="inlineStr">
         <is>
-          <t>CHK_014</t>
+          <t>CHK_018</t>
         </is>
       </c>
       <c r="F38" s="18" t="inlineStr">
         <is>
-          <t>TC_045,TC_054</t>
+          <t>TC_036</t>
         </is>
       </c>
     </row>
@@ -2757,12 +2757,12 @@
       </c>
       <c r="E39" s="18" t="inlineStr">
         <is>
-          <t>CHK_015</t>
+          <t>CHK_019</t>
         </is>
       </c>
       <c r="F39" s="18" t="inlineStr">
         <is>
-          <t>TC_052</t>
+          <t>TC_037</t>
         </is>
       </c>
     </row>
@@ -2791,12 +2791,12 @@
       </c>
       <c r="E40" s="18" t="inlineStr">
         <is>
-          <t>CHK_015</t>
+          <t>CHK_019</t>
         </is>
       </c>
       <c r="F40" s="18" t="inlineStr">
         <is>
-          <t>TC_052</t>
+          <t>TC_038</t>
         </is>
       </c>
     </row>
@@ -2825,12 +2825,12 @@
       </c>
       <c r="E41" s="18" t="inlineStr">
         <is>
-          <t>CHK_016</t>
+          <t>CHK_020</t>
         </is>
       </c>
       <c r="F41" s="18" t="inlineStr">
         <is>
-          <t>TC_043</t>
+          <t>TC_039</t>
         </is>
       </c>
     </row>
@@ -2859,12 +2859,12 @@
       </c>
       <c r="E42" s="18" t="inlineStr">
         <is>
-          <t>CHK_016</t>
+          <t>CHK_020</t>
         </is>
       </c>
       <c r="F42" s="18" t="inlineStr">
         <is>
-          <t>TC_042,TC_055</t>
+          <t>TC_040</t>
         </is>
       </c>
     </row>
@@ -2893,12 +2893,12 @@
       </c>
       <c r="E43" s="18" t="inlineStr">
         <is>
-          <t>CHK_016</t>
+          <t>CHK_020</t>
         </is>
       </c>
       <c r="F43" s="18" t="inlineStr">
         <is>
-          <t>TC_043</t>
+          <t>TC_039</t>
         </is>
       </c>
     </row>
@@ -2927,12 +2927,12 @@
       </c>
       <c r="E44" s="18" t="inlineStr">
         <is>
-          <t>CHK_016</t>
+          <t>CHK_020</t>
         </is>
       </c>
       <c r="F44" s="18" t="inlineStr">
         <is>
-          <t>TC_045</t>
+          <t>TC_040</t>
         </is>
       </c>
     </row>
@@ -2961,12 +2961,12 @@
       </c>
       <c r="E45" s="18" t="inlineStr">
         <is>
-          <t>CHK_016</t>
+          <t>CHK_021</t>
         </is>
       </c>
       <c r="F45" s="18" t="inlineStr">
         <is>
-          <t>TC_004</t>
+          <t>TC_041</t>
         </is>
       </c>
     </row>
@@ -2995,12 +2995,12 @@
       </c>
       <c r="E46" s="18" t="inlineStr">
         <is>
-          <t>CHK_015</t>
+          <t>CHK_022</t>
         </is>
       </c>
       <c r="F46" s="18" t="inlineStr">
         <is>
-          <t>TC_016,TC_037</t>
+          <t>TC_042</t>
         </is>
       </c>
     </row>
@@ -3029,12 +3029,12 @@
       </c>
       <c r="E47" s="18" t="inlineStr">
         <is>
-          <t>CHK_015</t>
+          <t>CHK_022</t>
         </is>
       </c>
       <c r="F47" s="18" t="inlineStr">
         <is>
-          <t>TC_017</t>
+          <t>TC_043</t>
         </is>
       </c>
     </row>
@@ -3063,12 +3063,12 @@
       </c>
       <c r="E48" s="18" t="inlineStr">
         <is>
-          <t>CHK_015</t>
+          <t>CHK_022</t>
         </is>
       </c>
       <c r="F48" s="18" t="inlineStr">
         <is>
-          <t>TC_019</t>
+          <t>TC_044</t>
         </is>
       </c>
     </row>
@@ -3097,12 +3097,12 @@
       </c>
       <c r="E49" s="18" t="inlineStr">
         <is>
-          <t>CHK_006</t>
+          <t>CHK_023</t>
         </is>
       </c>
       <c r="F49" s="18" t="inlineStr">
         <is>
-          <t>TC_027</t>
+          <t>TC_045</t>
         </is>
       </c>
     </row>
@@ -3131,12 +3131,12 @@
       </c>
       <c r="E50" s="18" t="inlineStr">
         <is>
-          <t>CHK_006</t>
+          <t>CHK_023</t>
         </is>
       </c>
       <c r="F50" s="18" t="inlineStr">
         <is>
-          <t>TC_028</t>
+          <t>TC_046</t>
         </is>
       </c>
     </row>
@@ -3411,17 +3411,17 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>reset_state_checker</t>
+          <t>clk_stability_checker</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>检查rst_ni异步复位及同步释放后模块状态正确性：
-1.复位后所有状态机回到IDLE态：front_state=IDLE，back_state=S_IDLE，axi_state=AXI_IDLE；
-2.复位后所有输出deassert：pdo_oe_o=0，htrans_o=2'b00(IDLE)，csr_rd_en_o=0，csr_wr_en_o=0；
-3.pdo_o[15:0]=16'b0，协议上下文清空；
-4.RX/TX FIFO清空：rxfifo_empty_o=1，txfifo_empty_o=1；
-5.CTRL.EN=0，CTRL.LANE_MODE=2'b00(1-bit默认)，LAST_ERR=0x00。</t>
+          <t>检查clk_i时钟稳定性和单时钟域正确性：
+1.clk_i频率稳定在100MHz±1%范围内，周期抖动不超过±1%；
+2.所有内部逻辑（协议采样、状态机、AHB-Lite Master）均在clk_i上升沿同步，不存在跨时钟域路径；
+3.AHB侧htrans_o[1:0]/hburst_o[2:0]/haddr_o[31:0]与协议侧pcs_n_i/pdi_i[15:0]/pdo_o[15:0]共用同一clk_i域；
+4.长时间运行（≥10µs）下clk_i周期无累积漂移；
+5.各lane_mode下bpc(bits per clock)计算与clk_i周期一致：1-bit=1bpc, 4-bit=4bpc, 8-bit=8bpc, 16-bit=16bpc。</t>
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
@@ -3434,16 +3434,18 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>clk_stability_checker</t>
+          <t>reset_state_checker</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>检查clk_i时钟域和频率正确性：
-1.clk_i目标频率100MHz，周期10ns，周期误差在±1%内（9.9ns~10.1ns）；
-2.模块采用单时钟域设计，AHB侧(htrans_o/haddr_o/hwdata_o/hrdata_i等)与协议侧(pdi_i[15:0]/pdo_o[15:0]/pdo_oe_o等)共用clk_i同域工作；
-3.所有内部寄存器在clk_i上升沿采样，无异步数据路径（rst_ni异步复位除外）；AHB 2-phase流水中地址相与数据相overlap 1拍均在clk_i上升沿同步；
-4.clk_i无毛刺，上升沿单周期有效；pdi_i[15:0]在有效周期内不得毛刺切换；pcs_n_i应满足建立保持要求。</t>
+          <t>检查rst_ni异步复位及同步释放后模块状态正确性：
+1.复位后所有状态机回到IDLE态：front_state=IDLE(3'd0), back_state=S_IDLE(3'd0), axi_state=AXI_IDLE(3'b000)；
+2.复位后所有输出deassert：pdo_oe_o=0, htrans_o[1:0]=2'b00(IDLE), csr_rd_en_o=0, csr_wr_en_o=0；
+3.pdo_o[15:0]=16'b0，协议上下文清空；
+4.RX/TX FIFO清空：rxfifo_empty_o=1, txfifo_empty_o=1；
+5.CTRL.EN=0, CTRL.LANE_MODE=2'b00(1-bit默认), LAST_ERR=0x00；
+6.Burst中途复位：所有FSM立即跳转IDLE，RXFIFO/TXFIFO强制drain至empty。</t>
         </is>
       </c>
       <c r="D4" s="4" t="n"/>
@@ -3456,16 +3458,16 @@
       </c>
       <c r="B5" s="33" t="inlineStr">
         <is>
-          <t>csr_access_checker</t>
+          <t>csr_rw_checker</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>检查CSR接口读写时序和地址范围正确性：
-1.CSR写操作：csr_wr_en_o为单周期脉冲，同一周期内csr_addr_o[7:0]和csr_wdata_o[31:0]有效，外部CSR File在该上升沿采样完成写入；
+          <t>检查CSR接口读写时序正确性：
+1.CSR写操作：csr_wr_en_o为单周期脉冲，同一周期内csr_addr_o[7:0]和csr_wdata_o[31:0]有效，外部CSR File在该clk上升沿采样完成写入；
 2.CSR读操作：csr_rd_en_o为单周期脉冲，外部CSR File在下一周期将读数据稳定在csr_rdata_i[31:0]，模块在该周期采样（1 cycle读延迟）；
 3.CSR有效地址范围0x00~0x3F，reg_addr&gt;=0x40的访问在前置检查阶段即被拒绝，返回STS_BAD_REG(0x10)，不出现csr_rd_en_o/csr_wr_en_o脉冲；
-4.寄存器属性正确：VERSION(0x00)为RO，CTRL(0x04)为RW，STATUS(0x08)为RO，LAST_ERR(0x0C)为RO，BURST_CNT(0x10)为WC（写1清零）。</t>
+4.寄存器属性正确：VERSION(0x00)为RO, CTRL(0x04)为RW, STATUS(0x08)为RO, LAST_ERR(0x0C)为RO, BURST_CNT(0x10)为WC。</t>
         </is>
       </c>
       <c r="D5" s="13" t="n"/>
@@ -3478,16 +3480,18 @@
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>mode_reject_checker</t>
+          <t>csr_register_attr_checker</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>检查test_mode_i与en_i前置拒绝行为和优先级正确性：
-1.test_mode_i=0时：所有命令被拒绝返回STS_NOT_IN_TEST(0x04)，不产生csr_wr_en_o/csr_rd_en_o/htrans_o脉冲；
-2.en_i=0时：所有命令被拒绝返回STS_DISABLED(0x08)，不产生csr_wr_en_o/csr_rd_en_o/htrans_o脉冲；
-3.test_mode_i=0且en_i=0同时不满足时：返回STS_NOT_IN_TEST(0x04)，优先级STS_NOT_IN_TEST(0x04)&gt;STS_DISABLED(0x08)；
-4.test_mode_i在frame_valid时刻被SLC_DPCHK组合采样。</t>
+          <t>检查CSR寄存器属性与地址映射正确性：
+1.VERSION(0x00)为RO：写入后读回值不变（仍为编译期固化常量）；
+2.CTRL(0x04)为RW：写入后读回值一致，字段EN/LANE_MODE[1:0]/SOFT_RST可独立配置；
+3.STATUS(0x08)为RO：硬件每拍/每事务更新，写入无效；位域BUSY[0]/RESP_VALID[1]/CMD_ERR[2]/BUS_ERR[3]/FRAME_ERR[4]/IN_TEST_MODE[5]/OUT_EN[6]/BURST_ERR[7]；
+4.LAST_ERR(0x0C)为RO(sticky)：错误发生时锁存错误码，软件通过BURST_CNT(0x10)WC语义间接清除不适用，LAST_ERR仅在新错误或复位时更新；
+5.BURST_CNT(0x10)为WC(≥16bit)：写1清零，读回当前Burst事务计数值；
+6.reg_addr&gt;=0x40返回STS_BAD_REG(0x10)，不产生csr_wr_en_o/csr_rd_en_o脉冲。</t>
         </is>
       </c>
       <c r="D6" s="13" t="n"/>
@@ -3500,16 +3504,17 @@
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>lane_mode_checker</t>
+          <t>test_mode_reject_checker</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>检查lane_mode_i对应的通道宽度和数据信号使用正确性：
-1.lane_mode_i=2'b00(1-bit模式)：仅使用pdi_i[0]/pdo_o[0]，pdi_i[15:1]忽略，pdo_o[15:1]驱动为0；RD_CSR帧16bit需16个周期接收；
-2.lane_mode_i=2'b01(4-bit模式)：使用pdi_i[3:0]/pdo_o[3:0]，按高nibble优先发送；RD_CSR帧16bit需4个周期接收；
-3.lane_mode_i=2'b10(8-bit模式)：使用pdi_i[7:0]/pdo_o[7:0]；lane_mode_i=2'b11(16-bit模式)：pdi_i[15:0]/pdo_o[15:0]全部有效；
-4.lane_mode_i在接收器(SLC_CAXIS)和发送器(SLC_SAXIS)中被连续组合采样，用于计算每拍移位宽度bpc(bits per clock)。</t>
+          <t>检查test_mode_i与en_i拒绝条件及优先级正确性：
+1.test_mode_i=0时：所有命令返回STS_NOT_IN_TEST(0x04)，不产生csr_wr_en_o/csr_rd_en_o/htrans_o脉冲；
+2.en_i=0时：所有命令返回STS_DISABLED(0x08)，不产生csr_wr_en_o/csr_rd_en_o/htrans_o脉冲；
+3.test_mode_i=0且en_i=0时：返回STS_NOT_IN_TEST(0x04)（优先级STS_NOT_IN_TEST(0x04) &gt; STS_DISABLED(0x08)）；
+4.SLC_DPCHK在frame_valid时刻组合采样test_mode_i与en_i，帧接收期间不影响接收过程；
+5.所有拒绝场景下AHB输出保持空闲：htrans_o[1:0]=2'b00(IDLE), hburst_o[2:0]=3'b000(SINGLE), haddr_o[31:0]=32'h0。</t>
         </is>
       </c>
       <c r="D7" s="13" t="n"/>
@@ -3522,16 +3527,18 @@
       </c>
       <c r="B8" s="33" t="inlineStr">
         <is>
-          <t>frame_protocol_checker</t>
+          <t>lane_mode_checker</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>检查类SPI帧协议时序和FIFO流控行为正确性：
-1.pcs_n_i=0开启帧接收，pdi_i[15:0]在请求阶段由ATE主机按MSB-first驱动；
-2.请求与响应之间固定插入1个clk_i周期turnaround，期间pdo_oe_o=0（HiZ态）；
-3.响应阶段pdo_oe_o=1拉高，模块驱动pdo_o[15:0]输出响应数据；Burst响应期间pdo_oe_o保持连续有效直至最后一个beat发送完成；
-4.RXFIFO满时rxfifo_full_o=1，SLC_CAXIS暂停接收（rx_shift_en=0）；TXFIFO空时txfifo_empty_o=1，SLC_SAXIS暂停移位但pdo_oe_o保持高电平。</t>
+          <t>检查lane_mode_i对应的通道宽度和数据信号使用正确性：
+1.lane_mode_i=2'b00(1-bit模式)：仅使用pdi_i[0]/pdo_o[0], pdi_i[15:1]忽略, pdo_o[15:1]驱动为0；RD_CSR帧16bit需16个周期接收；
+2.lane_mode_i=2'b01(4-bit模式)：使用pdi_i[3:0]/pdo_o[3:0], 按MSB-first发送；RD_CSR帧16bit需4个周期接收；
+3.lane_mode_i=2'b10(8-bit模式)：使用pdi_i[7:0]/pdo_o[7:0], RD_CSR帧16bit需2个周期接收；
+4.lane_mode_i=2'b11(16-bit模式)：使用pdi_i[15:0]/pdo_o[15:0], RD_CSR帧16bit需1个周期接收；
+5.lane_mode_i在接收器(SLC_CAXIS)和发送器(SLC_SAXIS)中被连续组合采样，用于计算每拍移位宽度bpc(bits per clock)；
+6.pcs_n_i=0期间lane_mode_i切换会导致rx_shift_q步进宽度立即改变，造成帧数据错位。</t>
         </is>
       </c>
       <c r="D8" s="13" t="n"/>
@@ -3544,16 +3551,18 @@
       </c>
       <c r="B9" s="33" t="inlineStr">
         <is>
-          <t>frame_format_checker</t>
+          <t>frame_protocol_checker</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>检查各类命令帧格式和响应长度正确性：
-1.六类命令帧长：WR_CSR=48bit(opcode8+reg_addr8+wdata32)，RD_CSR=16bit(opcode8+reg_addr8)，AHB_WR32=72bit(opcode8+addr32+wdata32)，AHB_RD32=40bit(opcode8+addr32)，AHB_WR_BURST=48+32·N bit，AHB_RD_BURST=48 bit请求；
-2.写命令响应8-bit(status)，Single读命令响应40-bit(status+rdata)，Burst读响应8+32·N bit，beat间无turnaround；
-3.所有协议字段按MSB-first传输；
-4.frame_valid在rx_count&gt;=expected_rx_bits时产生，寄存输出延迟1 cycle。</t>
+          <t>检查类SPI帧协议时序正确性：
+1.pcs_n_i拉低后模块开始接收请求，pcs_n_i=1表示空闲；
+2.请求与响应之间固定插入1个clk_i周期的turnaround，TA期间pdo_oe_o=0；
+3.响应阶段pdo_oe_o拉高，模块通过pdo_o[15:0]驱动响应数据（MSB-first）；
+4.写命令响应8bit(status only)，Single读命令响应40bit(status+rdata)，Burst读响应8+32·N bit；
+5.Burst读响应期间beat间无turnaround，pdo_oe_o保持连续有效直至最后一个beat发送完成；
+6.front_state在TX态(3'd4)时pdo_oe_o=1，在TX_BURST态(3'd5)时pdo_oe_o持续为1。</t>
         </is>
       </c>
       <c r="D9" s="13" t="n"/>
@@ -3571,12 +3580,12 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>检查Burst帧header解析和帧长修正正确性：
-1.Burst header格式：{opcode[7:0], burst_len[4:0], rsvd[2:0], addr[31:0]}共48-bit，位于opcode之后第2字节bits[7:3]为burst_len；
-2.合法burst_len取值{1,4,8,16}，其他值触发STS_BAD_BURST(0x80)；burst_len=1退化为SINGLE；
-3.前端两段式帧长解析：收满8-bit锁存opcode_latched_q确定初始expected_rx_bits；收满16-bit后对AHB_WR_BURST修正expected_rx_bits为48+32·burst_len，AHB_RD_BURST保持48-bit；
-4.AHB_WR_BURST的payload beat（每凑够32-bit）直接写入SLC_RXFIFO，不经过rx_shift_q[79:0]；
-5.rx_count_q[11:0]扩宽以容纳最大560-bit（48+32·16）Burst写帧长。</t>
+          <t>检查Burst帧接收与解码正确性：
+1.Burst header格式：{opcode[7:0], burst_len[4:0], rsvd[2:0], addr[31:0]}共48bit，收满8bit锁存opcode_latched_q，收满16bit后锁存burst_len_latched_q；
+2.AHB_WR_BURST(0x22)：收满16bit后修正expected_rx_bits为48+32·burst_len bit，payload beat推入SLC_RXFIFO；
+3.AHB_RD_BURST(0x23)：expected_rx_bits保持48bit不变，无payload接收；
+4.rx_count_q[11:0]&gt;=expected_rx_bits_q[11:0]时产生frame_valid（寄存输出延迟1 cycle）；
+5.接收阶段寄存器：rx_shift_q[79:0](header缓冲), rx_count_q[11:0], opcode_latched_q[7:0], burst_len_latched_q[4:0], expected_rx_bits_q[11:0], phase_q[1:0](IDLE/HEADER/PAYLOAD)。</t>
         </is>
       </c>
       <c r="D10" s="13" t="n"/>
@@ -3594,11 +3603,11 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>检查opcode译码正确性和非法opcode拒绝行为：
-1.合法opcode及译码：0x10(WR_CSR), 0x11(RD_CSR), 0x20(AHB_WR32), 0x21(AHB_RD32), 0x22(AHB_WR_BURST), 0x23(AHB_RD_BURST)，共6类；
-2.非法opcode（不在{0x10,0x11,0x20,0x21,0x22,0x23}中）由SLC_DPCHK前置检查拒绝，返回STS_BAD_OPCODE(0x02)；
-3.opcode在内部rx_shift_q[79:72]位置（左归一化后），前8-bit完成后锁存opcode_latched_q[7:0]；
-4.非法opcode不产生csr_rd_en_o/csr_wr_en_o/htrans_o脉冲。</t>
+          <t>检查opcode解码与非法opcode处理：
+1.6种合法opcode正确解码：0x10→WR_CSR(td_cmd_type=2'b00), 0x11→RD_CSR(td_cmd_type=2'b00), 0x20→AHB_WR32(td_cmd_type=2'b01), 0x21→AHB_RD32(td_cmd_type=2'b01), 0x22→AHB_WR_BURST(td_cmd_type=2'b10), 0x23→AHB_RD_BURST(td_cmd_type=2'b10)；
+2.非法opcode（不在{0x10,0x11,0x20,0x21,0x22,0x23}中）返回STS_BAD_OPCODE(0x02)；
+3.前端收满8bit后锁存opcode_latched_q，据此确定初始expected_rx_bits为对应帧长；
+4.BUS_OPCODE优先级低于FRAME_ERR(0x01)但高于NOT_IN_TEST(0x04)。</t>
         </is>
       </c>
       <c r="D11" s="13" t="n"/>
@@ -3611,16 +3620,17 @@
       </c>
       <c r="B12" s="33" t="inlineStr">
         <is>
-          <t>config_ctrl_checker</t>
+          <t>lane_switch_checker</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>检查CTRL寄存器配置和lane_mode切换约束正确性：
-1.CTRL寄存器(0x04)为RW属性，复位后镜像en_i/lane_mode_i/test_mode_i端口初值，端口为权威源；
-2.CTRL.EN镜像en_i端口，CTRL.LANE_MODE镜像lane_mode_i[1:0]；
-3.lane_mode_i在事务执行期(pcs_n_i=0期间)必须保持稳定，中途切换导致移位寄存器步进宽度bpc立即改变，帧数据错位；
-4.CTRL.SOFT_RST写1触发协议上下文清零并恢复默认lane模式(1-bit)；违反lane_mode稳定性的后果：可能误触发STS_BAD_OPCODE(0x02)或STS_FRAME_ERR(0x01)。</t>
+          <t>检查lane_mode切换约束与违规后果：
+1.pcs_n_i=1（空闲态）切换lane_mode_i：等待≥2 cycle同步后拉低pcs_n_i开始新事务，新事务按切换后lane模式执行；
+2.pcs_n_i=0（事务执行中）切换lane_mode_i：SLC_CAXIS/SLC_SAXIS中bpc立即改变，rx_shift_q步进宽度变化导致帧数据错位；
+3.违规后果：数据错位后opcode_latched_q可能为非法值→触发STS_BAD_OPCODE(0x02)，或rx_count与expected_rx_bits失配→触发STS_FRAME_ERR(0x01)；
+4.模块不检测此违规行为，由集成方保证lane_mode_i在pcs_n_i=0期间保持稳定；
+5.CTRL.LANE_MODE[1:0]在复位后镜像lane_mode_i端口初值，端口为权威源。</t>
         </is>
       </c>
       <c r="D12" s="13" t="n"/>
@@ -3633,16 +3643,18 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>status_report_checker</t>
+          <t>status_err_tracker_checker</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>检查STATUS/LAST_ERR寄存器状态报告和FIFO状态输出正确性：
-1.MVP版本不实现独立中断输出端口，所有错误与完成状态通过STATUS寄存器和LAST_ERR寄存器查询，由ATE主机轮询获取；
-2.STATUS寄存器(0x08)8-bit位域：BUSY[0], RESP_VALID[1], CMD_ERR[2](sticky), BUS_ERR[3](sticky), FRAME_ERR[4](sticky), IN_TEST_MODE[5], OUT_EN[6], BURST_ERR[7](sticky)；
-3.LAST_ERR寄存器(0x0C)为RO属性，保存最近一次错误码（sticky），由外部CSR File实现WC语义清除；
-4.FIFO状态通过rxfifo_empty_o/rxfifo_full_o/txfifo_empty_o/txfifo_full_o四个端口持续输出（组合输出）。</t>
+          <t>检查STATUS/LAST_ERR寄存器状态追踪正确性：
+1.STATUS[0]BUSY：当前有事务执行时为1，空闲时为0；
+2.STATUS[1]RESP_VALID：最近响应有效时置1；
+3.STATUS[2]CMD_ERR/STATUS[3]BUS_ERR/STATUS[4]FRAME_ERR/STATUS[7]BURST_ERR：sticky位，错误发生后保持直至软件清除；
+4.STATUS[5]IN_TEST_MODE：镜像test_mode_i；STATUS[6]OUT_EN：镜像pdo_oe_o；
+5.LAST_ERR[7:0]：保存最近一次错误码(sticky)，新错误覆盖旧值，复位清零；
+6.v2.2不实现独立中断输出端口(IRQ)，所有状态通过轮询STATUS/LAST_ERR获取。</t>
         </is>
       </c>
       <c r="D13" s="4" t="n"/>
@@ -3660,12 +3672,12 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>检查错误优先级链和执行期错误检测正确性：
-1.前置检查错误按固定优先级链返回(高→低)：STS_FRAME_ERR(0x01)&gt;STS_BAD_OPCODE(0x02)&gt;STS_NOT_IN_TEST(0x04)&gt;STS_DISABLED(0x08)&gt;STS_BAD_REG(0x10)&gt;STS_ALIGN_ERR(0x20)&gt;STS_BAD_BURST(0x80)&gt;STS_BURST_BOUND(0x81)；
+          <t>检查错误优先级链和多异常并发处理正确性：
+1.前置检查错误按固定优先级链返回(高→低)：STS_FRAME_ERR(0x01) &gt; STS_BAD_OPCODE(0x02) &gt; STS_NOT_IN_TEST(0x04) &gt; STS_DISABLED(0x08) &gt; STS_BAD_REG(0x10) &gt; STS_ALIGN_ERR(0x20) &gt; STS_BAD_BURST(0x80) &gt; STS_BURST_BOUND(0x81)；
 2.任何前置错误均在发起CSR/AHB访问前收敛，不产生csr_wr_en_o/csr_rd_en_o/htrans_o脉冲；
 3.STS_AHB_ERR(0x40)不在前置优先级链中：仅在前置检查全部通过后、AHB事务实际执行期间发生，与前置错误互斥；
-4.AHB执行期错误：hresp_i=1时返回STS_AHB_ERR(0x40)；hready_i持续为0超过BUS_TIMEOUT_CYCLES(256)周期触发超时（9-bit计数器，AXI_WAIT态每拍+1，计至255触发AXI_ERR），返回STS_AHB_ERR(0x40)；
-5.Burst内任一beat上hresp_i=1立即中止burst，进入AXI_ERR状态。</t>
+4.多个前置错误条件同时成立时，仅报告最高优先级的单个错误；
+5.SLC_DPCHK对frame_valid/frame_abort/opcode/test_mode_i/en_i/reg_addr/addr[1:0]/burst_len/addr[9:0]+4·(burst_len-1)进行组合逻辑检查。</t>
         </is>
       </c>
       <c r="D14" s="13" t="n"/>
@@ -3678,17 +3690,17 @@
       </c>
       <c r="B15" s="33" t="inlineStr">
         <is>
-          <t>burst_error_checker</t>
+          <t>align_err_checker</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>检查Burst参数前置检查和Burst执行期错误处理正确性：
-1.burst_len不在{1,4,8,16}中由SLC_DPCHK前置检查拒绝，返回STS_BAD_BURST(0x80)，不发起任何AHB事务；
-2.addr[9:0]+4·(burst_len-1)&gt;=1024判定跨1KB边界，返回STS_BURST_BOUND(0x81)，不发起任何AHB事务；
-3.Burst中途hresp_i=1：axi_state跳转AXI_ERR，剩余beat取消，返回STS_AHB_ERR(0x40)；
-4.TXFIFO中已缓冲的部分beat仍按正常路径发往前端，ATE收到的响应数据流可能短于burst_len拍；
-5.STS_BAD_BURST(0x80)和STS_BURST_BOUND(0x81)在优先级链中位于STS_ALIGN_ERR(0x20)之后。</t>
+          <t>检查AHB地址对齐错误检测：
+1.AHB命令addr[1:0]!=2'b00时返回STS_ALIGN_ERR(0x20)，不发起AHB访问；
+2.htrans_o[1:0]保持2'b00(IDLE)，不出现NONSEQ/SEQ脉冲；
+3.ALIGN_ERR(0x20)在优先级链中位于STS_BAD_REG(0x10)之后、STS_BAD_BURST(0x80)之前；
+4.AHB访问固定32-bit WORD宽度(hsize_o=3'b010)，不支持byte/halfword访问；
+5.haddr_o[1:0]在合法AHB事务中始终为2'b00。</t>
         </is>
       </c>
       <c r="D15" s="13" t="n"/>
@@ -3701,17 +3713,18 @@
       </c>
       <c r="B16" s="33" t="inlineStr">
         <is>
-          <t>low_power_checker</t>
+          <t>frame_abort_checker</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>检查空闲态和反压态动态翻转控制及门控行为正确性：
-1.pcs_n_i=1(空闲态)时，RX移位寄存器与RX反序列化逻辑不更新；
-2.非TX/TA态时，TX移位寄存器与TX序列化逻辑不翻转；
-3.AHB超时计数器仅在AXI_WAIT状态激活，STATE_REQ清零，STATE_WAIT每拍+1；
-4.RXFIFO空时后端BURST_LOOP写数据通道门控；TXFIFO空时前端TX Sequencer不启动；
-5.hburst_o在整个Burst期间保持稳定（不逐beat切换），避免组合逻辑翻转。</t>
+          <t>检查帧中止(frame_abort)检测与处理正确性：
+1.pcs_n_i在rx_count&lt;expected_rx_bits时提前拉高且opcode已锁存：产生frame_abort（寄存输出延迟1 cycle），返回STS_FRAME_ERR(0x01)；
+2.pcs_n_i在opcode锁存前(接收不足8bit)拉高：接收状态静默复位，不产生frame_abort，不返回任何状态码；
+3.FRAME_ERR(0x01)为最高优先级错误，不发起CSR/AHB访问；
+4.帧中止后前端FSM走IDLE→TA→TX(internal)错误返回路径；
+5.RXFIFO强制drain至empty；
+6.Burst payload接收中途pcs_n_i提前拉高：截断，返回STS_FRAME_ERR(0x01)，已推入RXFIFO的数据被drain，不发起AHB Burst。</t>
         </is>
       </c>
       <c r="D16" s="13" t="n"/>
@@ -3724,17 +3737,17 @@
       </c>
       <c r="B17" s="33" t="inlineStr">
         <is>
-          <t>ahb_master_checker</t>
+          <t>ahb_err_timeout_checker</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>检查AHB-Lite Master接口协议符合性和Burst时序正确性：
-1.hsize_o固定3'b010(WORD)，haddr_o[1:0]=2'b00(4-byte对齐)；
-2.htrans_o编码：IDLE=2'b00，NONSEQ=2'b10(首拍)，SEQ=2'b11(后续beat)；不支持BUSY传输类型；
-3.burst_len→hburst映射：1→SINGLE(3'b000)，4→INCR4(3'b011)，8→INCR8(3'b101)，16→INCR16(3'b111)；hburst_o在整个Burst期间保持稳定；
-4.AHB 2-phase流水：T1地址相(AXI_REQ)驱动haddr/hwrite/htrans=NONSEQ；T2数据相(AXI_WAIT)写驱动hwdata，读在hready_i=1时采样hrdata；地址相与数据相overlap 1拍；
-5.Burst内地址每拍自增+4，不支持WRAP Burst。</t>
+          <t>检查AHB错误响应与超时处理正确性：
+1.hresp_i=1在AXI_WAIT检测到时：axi_state跳转AXI_ERR(3'b101), err_o=1, 返回STS_AHB_ERR(0x40)；
+2.hready_i持续为0超过BUS_TIMEOUT_CYCLES(256)周期：timeout_cnt_q[8:0]递增至255(9-bit计数器), 触发AXI_ERR, 返回STS_AHB_ERR(0x40)；
+3.hresp错误与超时使用同一状态码STS_AHB_ERR(0x40)，不做区分；
+4.AXI_ERR下一拍自动转AXI_IDLE(3'b000)，AHB输出恢复空闲(htrans=IDLE, hburst=SINGLE, haddr=0)；
+5.Burst模式下每个beat独立计数超时，任一beat超时即中止整个burst。</t>
         </is>
       </c>
       <c r="D17" s="13" t="n"/>
@@ -3747,61 +3760,181 @@
       </c>
       <c r="B18" s="33" t="inlineStr">
         <is>
+          <t>burst_param_checker</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>检查Burst参数前置检查正确性：
+1.burst_len不在{1,4,8,16}中时返回STS_BAD_BURST(0x80)，不发起任何AHB访问，htrans_o保持IDLE；
+2.burst_len=1在RTL退化为SINGLE，等价于AHB_WR32/AHB_RD32；
+3.addr[9:0]+4·(burst_len-1)&gt;=1024时返回STS_BURST_BOUND(0x81)，不发起任何AHB访问；
+4.STS_BAD_BURST(0x80)和STS_BURST_BOUND(0x81)仅对AHB_WR_BURST(0x22)/AHB_RD_BURST(0x23)有效；
+5.BAD_BURST(0x80)和BURST_BOUND(0x81)在优先级链中位于ALIGN_ERR(0x20)之后，与AHB_ERR(0x40)互斥。</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>CHK_017</t>
+        </is>
+      </c>
+      <c r="B19" s="33" t="inlineStr">
+        <is>
+          <t>burst_mid_error_checker</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>检查Burst中途AHB错误处理正确性：
+1.Burst内任一beat上hresp_i=1：立即将FSM推入AXI_ERR(3'b101)，剩余beat不再发起，htrans_o跳转IDLE；
+2.已在TXFIFO中的部分beat仍会发往前端（ATE收到的响应数据流短于burst_len）；
+3.第N beat的X(invalid)数据不推入TXFIFO；
+4.Burst中途错误后RXFIFO/TXFIFO强制drain至empty；
+5.返回STS_AHB_ERR(0x40)，exec_status[7:0]=8'h40。</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>CHK_018</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>low_power_checker</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>检查空闲态翻转抑制和门控行为正确性：
+1.pcs_n_i=1时RX移位逻辑(rx_shift_q)和RX反序列化逻辑不更新；
+2.非TX/TA态时TX移位寄存器(tx_shift_q)和TX序列化逻辑不翻转；
+3.timeout_cnt_q仅在AXI_WAIT状态激活，其他状态不递增；
+4.test_mode_i=0或无有效任务时AHB输出保持空闲(htrans=IDLE, hburst=SINGLE, haddr=0)；
+5.RXFIFO写路径在rxfifo_empty_o=1时后端写入逻辑门控；TXFIFO读路径在txfifo_empty_o=1时前端TX Sequencer不启动；
+6.hburst_o[2:0]在整个Burst期间保持稳定，不逐beat切换。</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>CHK_019</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>perf_throughput_checker</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>检查Burst有效吞吐达标：
+1.AHB_WR_BURST×16在16-bit lane下：header 48bit(3拍RX)+payload 512bit(32拍RX)+AHB INCR16(16拍)+turnaround 1拍+status 8bit(1拍TX)≈54~56 cycles/64B，有效吞吐约116MB/s；
+2.AHB_RD_BURST×16在16-bit lane下：header 48bit(3拍RX)+AHB INCR16(17拍)+turnaround 1拍+response 520bit(33拍TX)≈54 cycles/64B，有效吞吐约118MB/s；
+3.1-bit lane下AHB_RD_BURST×16：约586 cycles，有效吞吐远低于16-bit lane；
+4.AHB zero-wait-state(hready_i=1)假设下延时最小，实际延时=基础延时+等待周期数；
+5.hsize_o[2:0]固定3'b010(WORD)，haddr_o[31:0]每beat自增+4。</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>CHK_020</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
           <t>dfx_stats_checker</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>检查DFX流量统计计数器和状态可观测点正确性：
-1.统计计数器（WC写1清零，各≥16bit）：每opcode成功次数6路(WR_CSR/RD_CSR/AHB_WR32/AHB_RD32/AHB_WR_BURST/AHB_RD_BURST)；每错误码失败次数8路(0x01/0x02/0x04/0x08/0x10/0x20/0x40/0x80)；
-2.CSR读/写次数各1路；AHB Single读/写次数各1路；Burst访问计数INCR4/8/16各读/写6路；
-3.total_burst_beat_cnt(≥24bit)每hready_i=1且state in {AXI_REQ,AXI_BURST,AXI_WAIT}时自增；rxfifo_backpressure_cnt在rxfifo_full_o上升沿累加；txfifo_stall_cnt在txfifo_full_o上升沿累加；
-4.可观测点：front_state_q[2:0], back_state_q[2:0], axi_state_q[2:0], rxfifo_cnt_o[5:0], txfifo_cnt_o[5:0], burst_beat_cnt_q[4:0], bus_timeout_cnt_q[8:0], last_err_q[7:0]；
-5.CSR自身不进入SoC AHB memory map，通过WR_CSR/RD_CSR协议命令访问。</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="33" t="n"/>
-      <c r="B19" s="33" t="n"/>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="13" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="33" t="n"/>
-      <c r="B20" s="33" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="13" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
-      <c r="C22" s="6" t="n"/>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>检查DFX统计计数器与可观测信号正确性：
+1.每opcode成功计数6路(WR_CSR/RD_CSR/AHB_WR32/AHB_RD32/AHB_WR_BURST/AHB_RD_BURST)：resp_valid&amp;&amp;status==STS_OK时自增，WC写1清零，位宽≥16bit；
+2.每错误码失败计数8路(0x01/0x02/0x04/0x08/0x10/0x20/0x40/0x80)：resp_valid&amp;&amp;status!=STS_OK时自增；
+3.Burst成功计数按hburst类型6路(INCR4/INCR8/INCR16各读/写)，total_burst_beat_cnt(≥24bit)，rxfifo_backpressure_cnt，txfifo_stall_cnt；
+4.FSM状态可观测：front_state_q[2:0]/back_state_q[2:0]/axi_state_q[2:0]通过STATUS_FSM寄存器(0x14地址段)以RO语义暴露；
+5.FIFO占用计数可观测：rxfifo_count_q[5:0]/txfifo_count_q[5:0]作为顶层输出。</t>
+        </is>
+      </c>
       <c r="D22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="6" t="n"/>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>CHK_021</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>memmap_checker</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>检查CSR与AHB memory map隔离正确性：
+1.模块自身CSR不进入SoC AHB memory map，通过WR_CSR/RD_CSR协议命令访问；
+2.AHB-Lite Master访问采用32bit地址空间和word访问粒度(hsize_o=3'b010)；
+3.具体可达目标地址范围由SoC顶层统一约束，模块本身不做无效地址判决；
+4.AHB侧对齐合法的地址是否落在有效memory map内由SoC AHB互联/解码器负责，返回hresp_i=1(含DECERR)时APLC-Lite统一映射为STS_AHB_ERR(0x40)。</t>
+        </is>
+      </c>
       <c r="D23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
-      <c r="C24" s="6" t="n"/>
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>CHK_022</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>ahb_protocol_checker</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>检查AHB-Lite Master 2-phase流水协议正确性：
+1.地址相：AXI_REQ态驱动htrans_o[1:0]=2'b10(NONSEQ) + haddr_o[31:0] + hwrite_o + hsize_o[2:0]=3'b010 + hburst_o[2:0]；
+2.Burst后续beat：AXI_BURST态驱动htrans_o=2'b11(SEQ), haddr_o每拍+4，hburst_o在整个burst期间保持稳定；
+3.数据相：写操作时hwdata_o[31:0]在地址相下一拍有效（与下一地址相overlap 1拍）；读操作时hrdata_i[31:0]在hready_i=1时采样；
+4.Burst结束：末beat htrans_o=2'b00(IDLE)，进入AXI_WAIT数据相，hready_i=1后转AXI_DONE；
+5.hburst映射：burst_len=1→SINGLE(3'b000), burst_len=4→INCR4(3'b011), burst_len=8→INCR8(3'b101), burst_len=16→INCR16(3'b111)。</t>
+        </is>
+      </c>
       <c r="D24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="n"/>
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="6" t="n"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>CHK_023</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>fifo_backpressure_checker</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>检查RXFIFO/TXFIFO反压与流控行为正确性：
+1.RXFIFO满(rxfifo_full_o=1)：SLC_CAXIS在PAYLOAD阶段暂停接收(不更新rx_shift_q/rxfifo_wr_en)，等待FIFO有空间后续接；
+2.RXFIFO反压期间rxfifo_count_q[5:0]在31/32间震荡（后端BURST_LOOP每cycle读1 word给hwdata_o时）；
+3.TXFIFO空(txfifo_empty_o=1)：SLC_SAXIS在TX_BURST阶段暂停移位，pdo_oe_o保持高电平(不释放总线方向), pdo_o[15:0]保持上一拍数据值；
+4.TXFIFO非空时立即恢复移位输出；
+5.FIFO深度默认32(FIFO_DEPTH参数化)，足以覆盖burst_len=16场景(16 beat+冗余)；
+6.FIFO空/满状态为组合输出(连续有效)，便于ATE或SoC观察。</t>
+        </is>
+      </c>
       <c r="D25" s="4" t="n"/>
     </row>
     <row r="26">
@@ -4047,19 +4180,21 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>验证clk_i时钟稳定性和单时钟域工作正确性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
-2.clk_i配置为100MHz(周期10ns)；
+          <t>配置条件：
+1.模块上电，clk_i稳定运行100MHz；
+2.test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
 输入激励：
-1.模块上电后运行1000个clk_i周期，执行AHB_RD32命令(opcode=0x21, addr=0x10000000)验证基本功能；
-2.执行AHB_RD_BURST×4命令(opcode=0x23, burst_len=4, addr=0x10000000)，持续运行10μs；
-3.测量clk_i周期统计，验证无周期抖动超限；
-4.验证AHB侧htrans_o与协议侧pdi_i/pdo_o同域工作，无异步数据路径；
+1.连续发送10条WR_CSR命令(opcode=0x10, reg_addr=0x04(CTRL), wdata递增0x01~0x0A)，每次pcs_n_i间隔≥2周期；
+2.切换lane_mode_i=2'b01(4-bit模式)，等待2周期同步；
+3.连续发送AHB_WR_BURST×4命令(opcode=0x22, burst_len=4, addr=0x20000000)，持续运行10µs；
+4.测量clk_i周期，计算周期误差；
+5.观察AHB侧htrans_o/hburst_o时序与协议侧pcs_n_i/pdi_i时序是否同域同步；
 期望结果：
-1.clk_i周期10ns±1%（9.9ns~10.1ns），无毛刺；
-2.所有命令正常完成，status_code=STS_OK(0x00)；
-3.AHB侧与协议侧信号同在clk_i上升沿采样，无跨域信号；
+1.clk_i频率稳定在100MHz±1%，周期抖动≤±1%；
+2.所有命令返回STS_OK(0x00)，无异常状态码；
+3.AHB输出与协议输出均与clk_i上升沿对齐，无跨域亚稳态；
+4.4-bit模式下持续运行10µs无功能异常；
+5.各lane_mode下bpc计算正确：1-bit=1bpc, 4-bit=4bpc, 16-bit=16bpc；
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
         </is>
@@ -4074,28 +4209,26 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>test_reset_behavior</t>
+          <t>test_async_reset</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>验证rst_ni异步复位、同步释放后模块恢复到正确初始状态。
-配置条件：
-1.模块上电，clk_i稳定运行100MHz；
-2.初始配置test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)；
+          <t>配置条件：
+1.模块上电，clk_i=100MHz；
+2.test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)；
 输入激励：
 1.拉低rst_ni触发异步复位（至少持续2个clk_i周期）；
-2.释放rst_ni（同步释放）；
-3.复位释放后发送RD_CSR命令(opcode=0x11, reg_addr=0x08读取STATUS寄存器)验证模块恢复工作；
-4.发送RD_CSR命令(opcode=0x11, reg_addr=0x04读取CTRL寄存器)验证复位值CTRL.EN=0, CTRL.LANE_MODE=2'b00；
-5.再次拉低rst_ni触发复位，释放后检查复位状态；
+2.释放rst_ni（同步释放，与clk_i上升沿对齐）；
+3.复位释放后发送RD_CSR命令(opcode=0x11, reg_addr=0x04(CTRL))验证模块恢复工作；
+4.发送RD_CSR命令(opcode=0x11, reg_addr=0x08(STATUS))检查复位默认值；
+5.再次拉低rst_ni触发复位，释放后检查所有FSM状态和输出信号；
 期望结果：
-1.复位后所有状态机回到IDLE态：front_state=IDLE，back_state=S_IDLE，axi_state=AXI_IDLE；
-2.输出信号deassert：pdo_oe_o=0，htrans_o=2'b00(IDLE)，csr_rd_en_o=0，csr_wr_en_o=0；
-3.pdo_o[15:0]=16'b0，协议上下文清空；
-4.RX/TX FIFO清空：rxfifo_empty_o=1，txfifo_empty_o=1；
-5.CTRL.EN=0，CTRL.LANE_MODE=2'b00(1-bit默认)；
-6.复位释放后RD_CSR命令正常响应status_code=STS_OK(0x00)；
+1.复位后所有状态机回到IDLE态：front_state=IDLE(3'd0), back_state=S_IDLE(3'd0), axi_state=AXI_IDLE(3'b000)；
+2.输出信号deassert：pdo_oe_o=0, htrans_o[1:0]=2'b00(IDLE), csr_rd_en_o=0, csr_wr_en_o=0；
+3.pdo_o[15:0]=16'b0；RX/TX FIFO清空：rxfifo_empty_o=1, txfifo_empty_o=1；
+4.CTRL.EN=0, CTRL.LANE_MODE=2'b00(1-bit默认)；
+5.复位释放后RD_CSR命令正常响应status_code=STS_OK(0x00)；
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
         </is>
@@ -4115,22 +4248,22 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>验证Burst执行中途异步复位立即终止所有操作并恢复初始状态。
-配置条件：
+          <t>配置条件：
 1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
-2.AHB zero-wait-state环境；
+2.AHB slave配置为正常响应(hready_i=1, hresp_i=0)；
 输入激励：
-1.发送AHB_RD_BURST×8命令(opcode=0x23, burst_len=8, addr=0x10000000)；
-2.等待axi_state=AXI_BURST（Burst执行中）；
-3.异步拉低rst_ni持续5个clk_i周期后同步释放；
-4.释放后发送RD_CSR命令(opcode=0x11, reg_addr=0x08)验证模块恢复；
+1.发送AHB_RD_BURST×8命令(opcode=0x23, burst_len=8, addr=0x20000000)；
+2.等待axi_state进入AXI_BURST(3'b010)，在第3个beat执行中异步拉低rst_ni；
+3.释放rst_ni（同步释放）；
+4.复位释放后发送RD_CSR命令(opcode=0x11, reg_addr=0x08(STATUS))验证模块恢复；
+5.发送WR_CSR命令(opcode=0x10, reg_addr=0x04(CTRL), wdata=0x00000001(CTRL.EN=1))恢复正常工作配置；
 期望结果：
-1.复位后所有FSM立即复位至IDLE：front_state=IDLE，back_state=S_IDLE，axi_state=AXI_IDLE；
-2.FIFO清空：rxfifo_empty_o=1，txfifo_empty_o=1；
-3.htrans_o=2'b00(IDLE)，pdo_oe_o=0；
-4.复位释放后模块可正常接受新命令，status_code=STS_OK(0x00)；
+1.复位立即生效：front_state=IDLE, back_state=S_IDLE, axi_state=AXI_IDLE；
+2.RXFIFO/TXFIFO强制drain至empty：rxfifo_empty_o=1, txfifo_empty_o=1；
+3.AHB输出恢复空闲：htrans_o=IDLE, hburst_o=SINGLE, haddr_o=0；
+4.复位释放后新命令正常响应STS_OK(0x00)；
 coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
+对axi_state各状态下的复位行为收集功能覆盖率</t>
         </is>
       </c>
       <c r="D5" s="13" t="n"/>
@@ -4148,1737 +4281,1701 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>验证CSR寄存器读写属性(RO/RW)的正确性，通过写-读序列证明属性。
-配置条件：
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1；
+2.lane_mode_i=2'b01(4-bit模式)；
+输入激励：
+1.发送WR_CSR命令：opcode=0x10, reg_addr=0x04(CTRL), wdata=0x00000001(CTRL.EN=1)；
+2.发送RD_CSR命令：opcode=0x11, reg_addr=0x04(CTRL)，验证RW寄存器写入后读回一致；
+3.发送RD_CSR命令：opcode=0x11, reg_addr=0x00(VERSION)，读取RO寄存器复位默认值；
+4.发送WR_CSR命令：opcode=0x10, reg_addr=0x00(VERSION), wdata=0xDEADBEEF（尝试写入RO寄存器）；
+5.发送RD_CSR命令：opcode=0x11, reg_addr=0x00(VERSION)，验证RO寄存器值未改变；
+6.发送RD_CSR命令：opcode=0x11, reg_addr=0x08(STATUS)，读取STATUS当前值；
+7.发送RD_CSR命令：opcode=0x11, reg_addr=0x0C(LAST_ERR)，读取LAST_ERR当前值；
+期望结果：
+1.WR+RD_CSR(CTRL)：写入0x01后读回0x00000001，证明RW属性——写入值可读回；
+2.RD_CSR(VERSION)：读回复位默认值（编译期固化常量）；
+3.WR+RD_CSR(VERSION)：尝试写入0xDEADBEEF后读回仍为复位默认值，证明RO属性——写入无效；
+4.RD_CSR(STATUS)：读回STATUS当前状态，STATUS[5]IN_TEST_MODE=1(test_mode_i=1), STATUS[6]OUT_EN=0(非发送)；
+5.RD_CSR(LAST_ERR)：读回0x00(无错误发生)；
+6.所有CSR读操作csr_rd_en_o产生单周期脉冲，下一周期csr_rdata_i有效；
+coverage check点：
+对CSR地址范围0x00/0x04/0x08/0x0C收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>TC_005</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>test_csr_bad_reg</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
 1.模块复位完成，test_mode_i=1，en_i=1；
 2.lane_mode_i=2'b11(16-bit模式)；
 输入激励：
-1.发送WR_CSR命令：opcode=0x10，reg_addr=0x04(CTRL)，wdata=0x00000001(CTRL.EN=1)；
-2.发送RD_CSR命令：opcode=0x11，reg_addr=0x04(CTRL)，验证RW寄存器写入后读回一致；
-3.发送WR_CSR命令：opcode=0x10，reg_addr=0x00(VERSION)，wdata=0xDEADBEEF（尝试写入RO寄存器）；
-4.发送RD_CSR命令：opcode=0x11，reg_addr=0x00(VERSION)，验证RO寄存器值未改变；
-5.发送WR_CSR命令：opcode=0x10，reg_addr=0x08(STATUS)，wdata=0xFFFFFFFF（尝试写入RO寄存器）；
-6.发送RD_CSR命令：opcode=0x11，reg_addr=0x08(STATUS)，验证RO寄存器值未改变；
-7.发送RD_CSR命令：opcode=0x11，reg_addr=0x0C(LAST_ERR)，验证RO寄存器可读；
+1.发送RD_CSR命令：opcode=0x11, reg_addr=0x40（超出0x00~0x3F范围的下边界外第1个地址）；
+2.发送WR_CSR命令：opcode=0x10, reg_addr=0xFF（最大非法地址），wdata=0x00000001；
+3.发送RD_CSR命令：opcode=0x11, reg_addr=0x3F（有效地址上界），验证合法访问；
+4.发送RD_CSR命令：opcode=0x11, reg_addr=0x00(VERSION)，验证前序非法访问未影响模块状态；
 期望结果：
-1.WR+RD_CSR(CTRL)：写入0x01后读回0x00000001，证明RW属性——写入值可读回；
-2.WR+RD_CSR(VERSION)：尝试写入0xDEADBEEF后读回仍为复位默认值，证明RO属性——写入无效；
-3.WR+RD_CSR(STATUS)：尝试写入0xFFFFFFFF后读回仍为复位默认值，证明RO属性——写入无效；
-4.所有CSR写操作：csr_wr_en_o为单周期脉冲，同一周期内csr_addr_o和csr_wdata_o有效；
-5.所有CSR读操作：csr_rd_en_o为单周期脉冲，下一周期csr_rdata_i有效（1 cycle读延迟）；
+1.reg_addr=0x40：返回STS_BAD_REG(0x10)，不产生csr_rd_en_o脉冲，htrans_o保持IDLE；
+2.reg_addr=0xFF：返回STS_BAD_REG(0x10)，不产生csr_wr_en_o脉冲；
+3.reg_addr=0x3F：正常访问返回STS_OK(0x00)，csr_rd_en_o产生单周期脉冲；
+4.前序非法访问后模块仍正常工作，VERSION读回值不受影响；
+5.BAD_REG(0x10)在优先级链中位于DISABLED(0x08)之后、ALIGN_ERR(0x20)之前；
 coverage check点：
-对CSR地址范围0x00~0x3F收集功能覆盖率，覆盖RW/RO属性验证场景</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TC_005</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>test_csr_bad_reg</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>验证非法CSR地址(reg_addr&gt;=0x40)被前置检查拒绝。
-配置条件：
+对reg_addr边界值(0x3F/0x40/0xFF)收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TC_006</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>test_burst_cnt_wc</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
 1.模块复位完成，test_mode_i=1，en_i=1；
 2.lane_mode_i=2'b11(16-bit模式)；
 输入激励：
-1.发送RD_CSR命令：opcode=0x11，reg_addr=0x40（超出0x00~0x3F范围）；
-2.发送RD_CSR命令：opcode=0x11，reg_addr=0x7F（远超范围）；
-3.发送WR_CSR命令：opcode=0x10，reg_addr=0x40，wdata=0x00000000（非法地址写）；
-4.发送RD_CSR命令：opcode=0x11，reg_addr=0x14（预留地址段0x14~0x1F，未实现）；
+1.发送RD_CSR命令：opcode=0x11, reg_addr=0x10(BURST_CNT)，读取复位后初始值（应为0）；
+2.执行3次AHB_RD_BURST×4命令(opcode=0x23, burst_len=4, addr=0x20000000)，每次成功；
+3.发送RD_CSR命令：opcode=0x11, reg_addr=0x10(BURST_CNT)，读取累加后值（应为3）；
+4.发送WR_CSR命令：opcode=0x10, reg_addr=0x10(BURST_CNT), wdata=0x00000001（写1清零）；
+5.发送RD_CSR命令：opcode=0x11, reg_addr=0x10(BURST_CNT)，验证WC清零成功（应回0）；
+6.发送WR_CSR命令：opcode=0x10, reg_addr=0x10(BURST_CNT), wdata=0x00000000（写0不清零）；
+7.执行1次AHB_RD_BURST×8命令，再RD_CSR(BURST_CNT)，验证写0不清零后计数正常累加；
 期望结果：
-1.reg_addr=0x40和0x7F返回STS_BAD_REG(0x10)，不产生csr_rd_en_o/csr_wr_en_o脉冲；
-2.reg_addr=0x40写操作同样返回STS_BAD_REG(0x10)，不产生csr_wr_en_o脉冲；
-3.所有非法地址访问均在前置检查阶段收敛，不发起CSR接口握手；
+1.复位后BURST_CNT=0x0000；
+2.3次Burst后BURST_CNT=0x0003；
+3.WC写1后BURST_CNT=0x0000，证明WC属性——写1清零；
+4.WC写0后BURST_CNT不变（写0不清零），新Burst后正常累加；
+5.BURST_CNT位宽≥16bit，短期不溢出；
 coverage check点：
-对CSR地址空间边界(0x3F/0x40)收集功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TC_006</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>test_burst_cnt_wc</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>验证BURST_CNT寄存器(0x10)的WC（写1清零）属性。
-配置条件：
+对BURST_CNT的WC属性验证场景收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>TC_007</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>test_test_mode_reject</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，lane_mode_i=2'b01(4-bit模式)；
+输入激励：
+1.设置test_mode_i=0，en_i=1；
+2.发送RD_CSR命令：opcode=0x11, reg_addr=0x00(VERSION)；
+3.检查响应帧status_code；
+4.复位模块，设置test_mode_i=1，en_i=0；
+5.发送WR_CSR命令：opcode=0x10, reg_addr=0x04(CTRL), wdata=0x01；
+6.检查响应帧status_code；
+7.复位模块，设置test_mode_i=0，en_i=0（同时不满足）；
+8.发送RD_CSR命令：opcode=0x11, reg_addr=0x00；
+9.检查响应帧status_code；
+期望结果：
+1.test_mode_i=0时：返回STS_NOT_IN_TEST(0x04)，不发起CSR/AHB访问，csr_rd_en_o=0；
+2.en_i=0时：返回STS_DISABLED(0x08)，不发起CSR/AHB访问，csr_wr_en_o=0, htrans_o=IDLE；
+3.test_mode_i=0且en_i=0时：返回STS_NOT_IN_TEST(0x04)（优先级STS_NOT_IN_TEST &gt; STS_DISABLED）；
+4.所有拒绝场景下htrans_o[1:0]=2'b00(IDLE)；
+coverage check点：
+对test_mode_i和en_i的组合状态(0/0, 0/1, 1/0)收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TC_008</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>test_en_disabled</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，lane_mode_i=2'b11(16-bit模式)；
+输入激励：
+1.设置en_i=0；
+2.发送AHB_RD32命令：opcode=0x21, addr=0x20000000；
+3.检查响应帧status_code和AHB输出；
+4.设置en_i=1；
+5.发送AHB_RD32命令：opcode=0x21, addr=0x20000000；
+6.检查响应帧status_code（验证恢复正常）；
+7.设置en_i=0后发送AHB_WR_BURST×4命令：opcode=0x22, burst_len=4, addr=0x20000000；
+期望结果：
+1.en_i=0时AHB_RD32返回STS_DISABLED(0x08)，不发起AHB访问，htrans_o保持IDLE；
+2.en_i=1时AHB_RD32正常返回STS_OK(0x00)，hrdata_i被正确采样；
+3.en_i=0时AHB_WR_BURST返回STS_DISABLED(0x08)，不发起任何AHB beat；
+4.DISABLED(0x08)优先级低于NOT_IN_TEST(0x04)但高于BAD_REG(0x10)；
+coverage check点：
+对en_i状态(0/1)×opcode类型收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>TC_009</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>test_mode_priority</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，lane_mode_i=2'b11(16-bit模式)；
+输入激励：
+1.设置test_mode_i=0，en_i=0；
+2.发送WR_CSR命令：opcode=0x10, reg_addr=0x04(CTRL), wdata=0x01；
+3.记录status_code；
+4.设置test_mode_i=0，en_i=1；
+5.发送WR_CSR命令：opcode=0x10, reg_addr=0x04(CTRL), wdata=0x01；
+6.记录status_code；
+7.对比步骤3与步骤6的status_code是否一致（均为STS_NOT_IN_TEST）；
+8.设置test_mode_i=1，en_i=0；
+9.发送WR_CSR命令，记录status_code（应为STS_DISABLED）；
+期望结果：
+1.test_mode_i=0且en_i=0：返回STS_NOT_IN_TEST(0x04)；
+2.test_mode_i=0且en_i=1：返回STS_NOT_IN_TEST(0x04)（优先级NOT_IN_TEST &gt; DISABLED）；
+3.test_mode_i=1且en_i=0：返回STS_DISABLED(0x08)；
+4.三种场景均不发起CSR/AHB访问：csr_wr_en_o=0, csr_rd_en_o=0, htrans_o=IDLE；
+5.证明优先级链STS_NOT_IN_TEST(0x04) &gt; STS_DISABLED(0x08)；
+coverage check点：
+对test_mode_i×en_i交叉覆盖收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC_010</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>test_1bit_lane</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1；
+2.lane_mode_i=2'b00(1-bit模式)；
+输入激励：
+1.通过pdi_i[0]按MSB-first顺序发送WR_CSR帧(opcode=0x10, reg_addr=0x04, wdata=0x00000001)，每拍1bit，共48拍；
+2.验证pdi_i[15:1]在接收期间被忽略（改变pdi_i[15:1]不影响接收结果）；
+3.发送RD_CSR帧(opcode=0x11, reg_addr=0x04)，共16拍，观察pdo_o[0]输出；
+4.检查pdo_o[15:1]是否驱动为0；
+5.测量接收阶段周期数是否为48拍(48bit/1bpc)；
+期望结果：
+1.WR_CSR接收48拍完成，frame_valid延迟1周期拉高；
+2.pdi_i[15:1]变化不影响接收正确性；
+3.RD_CSR响应在pdo_o[0]输出40bit(8bit status+32bit rdata)，pdo_o[15:1]=15'b0；
+4.rx_count_q每拍+1(1bpc)，接收阶段共48拍；
+5.status_code=STS_OK(0x00)；
+coverage check点：
+覆盖lane_mode_cp: lane_1bit bin</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC_011</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>test_4bit_lane</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1；
+2.lane_mode_i=2'b01(4-bit模式)；
+输入激励：
+1.通过pdi_i[3:0]按MSB-first顺序发送WR_CSR帧(opcode=0x10, reg_addr=0x04, wdata=0x00000001)，每拍4bit，共12拍；
+2.验证pdi_i[15:4]在接收期间被忽略；
+3.发送RD_CSR帧(opcode=0x11, reg_addr=0x04)，共4拍，观察pdo_o[3:0]输出；
+4.检查pdo_o[15:4]是否驱动为0；
+5.测量接收阶段周期数是否为12拍(48bit/4bpc)；
+期望结果：
+1.WR_CSR接收12拍完成(48bit/4bpc)；
+2.pdi_i[15:4]变化不影响接收正确性；
+3.RD_CSR响应在pdo_o[3:0]输出，pdo_o[15:4]=12'b0；
+4.rx_count_q每拍+4(4bpc)；
+5.status_code=STS_OK(0x00)，参考LRS §4.8.11；
+coverage check点：
+覆盖lane_mode_cp: lane_4bit bin</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC_012</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>test_8bit_lane</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1；
+2.lane_mode_i=2'b10(8-bit模式)；
+输入激励：
+1.通过pdi_i[7:0]按MSB-first顺序发送WR_CSR帧(opcode=0x10, reg_addr=0x04, wdata=0x00000001)，每拍8bit，共6拍；
+2.验证pdi_i[15:8]在接收期间被忽略；
+3.发送AHB_RD32帧(opcode=0x21, addr=0x20000000)，共5拍(40bit/8bpc)，观察pdo_o[7:0]输出；
+4.检查pdo_o[15:8]是否驱动为0；
+5.测量接收阶段周期数；
+期望结果：
+1.WR_CSR接收6拍完成(48bit/8bpc)；
+2.pdi_i[15:8]变化不影响接收正确性；
+3.AHB_RD32响应在pdo_o[7:0]输出40bit(8+32)，pdo_o[15:8]=8'b0；
+4.rx_count_q每拍+8(8bpc)；
+5.status_code=STS_OK(0x00)；
+coverage check点：
+覆盖lane_mode_cp: lane_8bit bin</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>TC_013</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>test_16bit_lane</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
 1.模块复位完成，test_mode_i=1，en_i=1；
 2.lane_mode_i=2'b11(16-bit模式)；
 输入激励：
-1.发送AHB_RD_BURST×4命令(opcode=0x23, burst_len=4, addr=0x10000000)使BURST_CNT递增；
-2.发送RD_CSR命令(opcode=0x11, reg_addr=0x10)读取BURST_CNT值，记录为cnt_before；
-3.再执行一条AHB_WR_BURST×4命令(opcode=0x22, burst_len=4, addr=0x20000000, wdata=4beat)；
-4.发送RD_CSR命令(opcode=0x11, reg_addr=0x10)读取BURST_CNT值，验证递增(cnt_after&gt;cnt_before)；
-5.发送WR_CSR命令(opcode=0x10, reg_addr=0x10, wdata=0x00000001)写1清零；
-6.发送RD_CSR命令(opcode=0x11, reg_addr=0x10)读回验证BURST_CNT=0x0000；
-7.发送WR_CSR命令(opcode=0x10, reg_addr=0x10, wdata=0x00000002)写非1值，验证WC属性——仅写1清零；
+1.通过pdi_i[15:0]按MSB-first顺序发送WR_CSR帧(opcode=0x10, reg_addr=0x04, wdata=0x00000001)，每拍16bit，共3拍；
+2.验证pdi_i[15:0]全部有效参与接收；
+3.发送AHB_RD32帧(opcode=0x21, addr=0x20000000)，共3拍(40bit/16bpc=3拍向上取整)；
+4.观察pdo_o[15:0]全部有效输出；
+5.测量接收和发送阶段周期数；
 期望结果：
-1.执行Burst后BURST_CNT非零且递增，证明计数功能正常；
-2.写1后BURST_CNT=0x0000，证明WC属性——写1清零生效；
-3.写非1值(0x02)后BURST_CNT仍为0x0000（已清零状态不变），或根据实现不清零，证明仅写1触发清零；
-4.所有CSR读写时序正确：csr_wr_en_o/csr_rd_en_o单周期脉冲；
+1.WR_CSR接收3拍完成(48bit/16bpc)；
+2.pdi_i[15:0]全部有效参与接收，rx_shift_q步进宽度16bpc；
+3.AHB_RD32响应在pdo_o[15:0]输出40bit(3拍TX，末拍8bit有效+8bit填充)；
+4.rx_count_q每拍+16(16bpc)；
+5.status_code=STS_OK(0x00)，参考LRS §4.8.2/§4.8.5；
+coverage check点：
+覆盖lane_mode_cp: lane_16bit bin</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC_014</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>test_wr_csr_protocol</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.pcs_n_i初始为高电平；
+输入激励：
+1.拉低pcs_n_i开始帧传输，按MSB-first顺序通过pdi_i[15:0]发送WR_CSR帧(opcode=0x10+reg_addr=0x04+wdata=0x00000001)；
+2.观察frame_valid延迟1周期拉高；
+3.观察csr_wr_en_o产生单周期脉冲，同一周期csr_addr_o[7:0]=0x04, csr_wdata_o[31:0]=0x00000001；
+4.观察turnaround 1周期(pdo_oe_o=0)；
+5.观察响应发送阶段pdo_oe_o=1，pdo_o[15:0]输出STS_OK(0x00)状态码；
+期望结果：
+1.frame_valid延迟1周期拉高（寄存输出）；
+2.csr_wr_en_o单周期脉冲，同周期csr_addr_o/csr_wdata_o有效；
+3.front_state经历IDLE→ISSUE→WAIT_RESP→TA→TX→IDLE完整流程；
+4.1周期turnaround，pdo_oe_o在TX态拉高；
+5.status_code=STS_OK(0x00)，参考LRS §4.8.2；
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>TC_007</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>test_mode_rejection</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>验证test_mode_i和en_i的拒绝行为和优先级，通过单条件+组合条件证明优先级链。
-配置条件：
-1.模块复位完成，lane_mode_i=2'b01(4-bit模式)；
+      <c r="D16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>TC_015</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>test_4bit_wr_csr</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b01(4-bit模式)；
+2.pcs_n_i初始为高电平；
 输入激励：
-1.设置test_mode_i=0，en_i=1；
-2.发送RD_CSR命令：opcode=0x11，reg_addr=0x00；
-3.检查响应帧status_code；
-4.复位模块，设置test_mode_i=1，en_i=0；
-5.发送WR_CSR命令：opcode=0x10，reg_addr=0x04，wdata=0x01；
-6.检查响应帧status_code；
-7.复位模块，设置test_mode_i=0，en_i=0（同时不满足）；
-8.发送RD_CSR命令：opcode=0x11，reg_addr=0x00；
-9.检查响应帧status_code；
+1.通过pdi_i[3:0]发送WR_CSR帧(opcode=0x10+reg_addr=0x04+wdata=0x00000001)，共12拍(48bit/4bpc)；
+2.观察接收阶段12拍完成；
+3.观察csr_wr_en_o脉冲和csr_addr_o/csr_wdata_o有效性；
+4.观察turnaround 1周期和响应发送2拍(8bit status/4bpc=2拍)；
+5.验证pdo_oe_o在TX期间=1；
 期望结果：
-1.test_mode_i=0时：返回STS_NOT_IN_TEST(0x04)，不发起CSR/AHB访问；
-2.en_i=0时：返回STS_DISABLED(0x08)，不发起CSR/AHB访问；
-3.test_mode_i=0且en_i=0时：返回STS_NOT_IN_TEST(0x04)（优先级STS_NOT_IN_TEST(0x04)&gt;STS_DISABLED(0x08)）；
-4.所有拒绝场景下csr_wr_en_o=0，csr_rd_en_o=0，htrans_o=IDLE；
+1.接收12拍(48bit/4bpc)，frame_valid延迟1周期拉高；
+2.csr_wr_en_o单周期脉冲，写入CTRL.EN=1；
+3.1周期turnaround后pdo_oe_o拉高，响应2拍输出STS_OK(0x00)；
+4.4-bit模式总耗时约17 cycles，参考LRS §4.8.11；
+5.front_state完整流程IDLE→ISSUE→WAIT_RESP→TA→TX→IDLE；
 coverage check点：
-对test_mode_i和en_i的组合状态收集功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>TC_008</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>test_1bit_lane</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>验证1-bit lane模式下数据收发正确性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b00(1-bit模式)；
+覆盖lane_mode_cp: lane_4bit bin, opcode_cp: wr_csr bin</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>TC_016</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>test_rd_csr_protocol</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
 输入激励：
-1.通过pdi_i[0]按MSB-first逐位发送WR_CSR帧(opcode=0x10, reg_addr=0x04, wdata=0x00000001)，共48bit=48拍；
-2.验证pdi_i[15:1]在1-bit模式下被忽略（驱动随机值不影响接收）；
-3.等待1 cycle turnaround，观察响应发送8bit=8拍通过pdo_o[0]输出；
-4.发送RD_CSR命令(opcode=0x11, reg_addr=0x04)，观察16bit RX=16拍，40bit TX=40拍；
-5.验证pdo_o[15:1]在响应阶段驱动为0；
+1.发送RD_CSR帧(opcode=0x11, reg_addr=0x00(VERSION))，请求帧16bit=1拍RX；
+2.观察csr_rd_en_o单周期脉冲，同周期csr_addr_o[7:0]=0x00；
+3.观察下一周期csr_rdata_i[31:0]有效（1 cycle读延迟）；
+4.观察1周期turnaround后pdo_oe_o拉高；
+5.观察响应帧40bit=3拍TX(status[7:0]+rdata[31:0])；
 期望结果：
-1.48拍接收完成，frame_valid延迟1 cycle拉高；
-2.pdo_o[0]输出status，pdo_o[15:1]=0；
-3.返回STS_OK(0x00)；
-4.RD_CSR读回CTRL=0x00000001，数据正确；
+1.请求1拍RX(16bit/16bpc)，frame_valid延迟1周期；
+2.csr_rd_en_o单周期脉冲，下一拍csr_rdata_i有效；
+3.front_state: IDLE→ISSUE→WAIT_RESP→TA→TX→IDLE；
+4.1周期turnaround，3拍TX输出status(0x00)+VERSION值；
+5.status_code=STS_OK(0x00)，参考LRS §4.8.3；
+coverage check点：
+覆盖opcode_cp: rd_csr bin</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>TC_017</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_wr32_protocol</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave配置为正常响应(hready_i=1, hresp_i=0)；
+输入激励：
+1.发送AHB_WR32帧(opcode=0x20, addr=0x20000000, wdata=0xCAFEBABE)，请求帧72bit=5拍RX；
+2.观察axi_state: AXI_IDLE→AXI_REQ→AXI_WAIT→AXI_DONE→AXI_IDLE；
+3.验证AXI_REQ态htrans_o=2'b10(NONSEQ), haddr_o=0x20000000, hwrite_o=1, hburst_o=3'b000(SINGLE)；
+4.验证AXI_WAIT态下一拍hwdata_o=0xCAFEBABE（数据相）；
+5.观察1周期turnaround和1拍TX响应(status=0x00)；
+期望结果：
+1.请求5拍RX(72bit/16bpc=5拍)，frame_valid延迟1周期；
+2.AHB 2-phase: T1地址相(NONSEQ+haddr), T2数据相(hwdata)；
+3.hsize_o[2:0]=3'b010(WORD), hwrite_o=1；
+4.status_code=STS_OK(0x00)，参考LRS §4.8.4；
+5.1拍TX输出8bit status；
+coverage check点：
+覆盖opcode_cp: ahb_wr32 bin, axi_fsm_cp各状态</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>TC_018</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_rd32_protocol</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave配置为正常响应(hready_i=1, hresp_i=0, hrdata_i=0xDEADBEEF)；
+输入激励：
+1.发送AHB_RD32帧(opcode=0x21, addr=0x20000000)，请求帧40bit=3拍RX；
+2.观察axi_state: AXI_IDLE→AXI_REQ→AXI_WAIT→AXI_DONE→AXI_IDLE；
+3.验证AXI_REQ态htrans_o=2'b10(NONSEQ), haddr_o=0x20000000, hwrite_o=0, hburst_o=SINGLE；
+4.验证AXI_WAIT态hready_i=1时采样hrdata_i=0xDEADBEEF；
+5.观察1周期turnaround和3拍TX响应(status+0xDEADBEEF)；
+期望结果：
+1.请求3拍RX(40bit/16bpc)，frame_valid延迟1周期；
+2.htrans_o: IDLE→NONSEQ→IDLE，hsize_o=3'b010(WORD)；
+3.hrdata_i在AXI_WAIT态被采样；
+4.3拍TX输出status(0x00)+rdata(0xDEADBEEF)；
+5.参考LRS §4.8.5/§4.8.1时序完全一致；
+coverage check点：
+覆盖opcode_cp: ahb_rd32 bin, axi_fsm_cp: AXI_REQ/AXI_WAIT/AXI_DONE</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TC_019</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_rd_burst4</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave配置为正常响应(hready_i=1, hresp_i=0, hrdata_i按beat递增D0/D1/D2/D3)；
+输入激励：
+1.发送AHB_RD_BURST×4帧(opcode=0x23, burst_len=4, addr=0x20000000)，请求帧48bit=3拍RX；
+2.观察task_req/task_ack一拍握手；
+3.验证hburst_o=INCR4(3'b011)保持稳定，htrans_o: NONSEQ→SEQ×3→IDLE，haddr每拍+4；
+4.验证4个beat hrdata_i=D0/D1/D2/D3被正确采样并推入TXFIFO；
+5.观察1周期turnaround后9拍TX(8+32×4=136bit/16bpc=9拍)输出status+rdata×4；
+期望结果：
+1.axi_state: AXI_IDLE→AXI_REQ→AXI_BURST→AXI_WAIT→AXI_DONE→AXI_IDLE；
+2.hburst_o=INCR4(3'b011)在整个burst期间稳定；
+3.resp_last在第4 beat置位；
+4.Burst读响应beat间无turnaround，pdo_oe_o持续为1；
+5.status_code=STS_OK(0x00)，参考LRS §4.8.6；
+coverage check点：
+覆盖burst_len_cp: incr4 bin, axi_fsm_cp: AXI_BURST</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TC_020</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_rd_burst8</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave正常响应(hready_i=1, hresp_i=0, hrdata_i按beat递增D0~D7)；
+输入激励：
+1.发送AHB_RD_BURST×8帧(opcode=0x23, burst_len=8, addr=0x20000000)，请求帧48bit=3拍RX；
+2.验证rx_count_q: 0→16→32→48, frame_valid在48bit满后脉冲；
+3.验证hburst_o=INCR8(3'b101)保持稳定，htrans_o: NONSEQ→SEQ×7→IDLE，haddr: A/A+4/.../A+0x1C；
+4.验证8个beat hrdata_i=D0~D7被正确采样，resp_last在第8 beat置位；
+5.观察1周期turnaround后TX输出status+rdata×8(8+256=264bit/16bpc=17拍TX)；
+期望结果：
+1.axi_state: AXI_IDLE→AXI_REQ→AXI_BURST→AXI_WAIT→AXI_DONE→AXI_IDLE完整流转；
+2.hburst_o=INCR8(3'b101)在整个burst地址相期间保持稳定；
+3.8个beat连续采样hrdata_i，全部推入TXFIFO；
+4.Burst读响应17拍TX，beat间无turnaround；
+5.status_code=STS_OK(0x00)，参考LRS §4.8.7；
+coverage check点：
+覆盖burst_len_cp: incr8 bin, opcode_cp: ahb_rd_burst bin</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TC_021</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_wr_burst4</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave正常响应(hready_i=1, hresp_i=0)；
+输入激励：
+1.发送AHB_WR_BURST×4帧(opcode=0x22, burst_len=4, addr=0x20000000)，Header 48bit=3拍RX，Payload 4×32bit=8拍RX，数据推入RXFIFO；
+2.观察rxfifo_wr_en在Payload阶段每2拍产生1次(32bit/16bpc)；
+3.验证hburst_o=INCR4(3'b011), htrans_o: NONSEQ→SEQ×3→IDLE, hwrite_o=1；
+4.验证后端从RXFIFO读出D0/D1/D2/D3作为hwdata_o输出；
+5.观察1周期turnaround和1拍TX响应(status)；
+期望结果：
+1.Header 3拍+Payload 8拍=11拍RX，frame_valid延迟1周期；
+2.RXFIFO正常缓冲4个beat数据，rxfifo_rd_en在BURST_LOOP期间触发；
+3.hwdata_o依次输出D0/D1/D2/D3，与AHB 2-phase流水对齐；
+4.back_state: S_IDLE→S_LOAD_TASK→S_EXEC→S_BURST_LOOP→S_BUILD_RESP→S_DONE→S_IDLE；
+5.status_code=STS_OK(0x00)，参考LRS §4.8.8；
+coverage check点：
+覆盖burst_len_cp: incr4 bin, opcode_cp: ahb_wr_burst bin, back_fsm_cp: S_BURST_LOOP</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TC_022</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>test_bad_opcode</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+输入激励：
+1.发送opcode=0xFF的命令帧（非法opcode），观察frame_valid和opcode_latched_q；
+2.发送opcode=0x00的命令帧（非法opcode，在合法范围外）；
+3.发送opcode=0x24的命令帧（紧邻合法范围0x23之后的非法值）；
+4.发送opcode=0x0F的命令帧（低半段非法值）；
+5.每次检查返回的status_code和AHB/CSR接口信号；
+期望结果：
+1.所有非法opcode返回STS_BAD_OPCODE(0x02)；
+2.不产生csr_wr_en_o/csr_rd_en_o脉冲，不产生htrans_o NSEQ/SEQ脉冲；
+3.BAD_OPCODE(0x02)优先级低于FRAME_ERR(0x01)但高于NOT_IN_TEST(0x04)；
+4.前端FSM走IDLE→TA→TX错误返回路径；
+5.LAST_ERR[7:0]被更新为0x02(sticky)；
+coverage check点：
+覆盖opcode_cp: illegal bin, status_cp: bad_opcode bin</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TC_023</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>test_all_opcode_legal</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave正常响应；
+输入激励：
+1.发送WR_CSR(opcode=0x10, reg_addr=0x04, wdata=0x01)，检查返回STS_OK；
+2.发送RD_CSR(opcode=0x11, reg_addr=0x00)，检查返回STS_OK+rdata；
+3.发送AHB_WR32(opcode=0x20, addr=0x20000000, wdata=0x12345678)，检查返回STS_OK；
+4.发送AHB_RD32(opcode=0x21, addr=0x20000000)，检查返回STS_OK+rdata；
+5.发送AHB_WR_BURST(opcode=0x22, burst_len=4, addr=0x20000000, wdata×4)，检查返回STS_OK；
+6.发送AHB_RD_BURST(opcode=0x23, burst_len=4, addr=0x20000000)，检查返回STS_OK+rdata×4；
+期望结果：
+1.6种opcode全部正确解码，td_cmd_type/td_is_read/td_burst_len正确设置；
+2.WR_CSR/RD_CSR走CSR路径，AHB命令走AXI路径；
+3.Burst命令td_burst_len和td_hburst正确映射；
+4.所有命令返回STS_OK(0x00)；
+5.6种opcode的CSR/AHB接口信号均符合预期时序；
+coverage check点：
+覆盖opcode_cp所有6个legal bins</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TC_024</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>test_lane_switch_idle</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.pcs_n_i=1（空闲态）；
+输入激励：
+1.在pcs_n_i=1期间切换lane_mode_i从2'b11(16-bit)→2'b00(1-bit)；
+2.等待≥2周期同步；
+3.拉低pcs_n_i开始新事务，通过pdi_i[0]发送WR_CSR帧(48拍/1bpc)；
+4.验证接收按1-bit模式执行(48拍)；
+5.切换lane_mode_i从2'b00→2'b01(4-bit)，等待2周期，再执行RD_CSR帧(4拍/4bpc)；
+期望结果：
+1.16-bit→1-bit切换成功，新事务按1-bit模式执行，rx_count_q每拍+1；
+2.pdi_i[0]有效，pdi_i[15:1]忽略；
+3.1-bit→4-bit切换成功，新事务按4-bit模式执行，rx_count_q每拍+4；
+4.两次事务均返回STS_OK(0x00)；
+5.CTRL.LANE_MODE[1:0]在事务后正确镜像新lane_mode_i值；
+coverage check点：
+覆盖lane_mode_cp: lane_1bit和lane_4bit bin切换场景</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TC_025</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>test_lane_switch_during_txn</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.pcs_n_i=0（事务进行中），AHB slave正常响应；
+输入激励：
+1.发送WR_CSR帧(pdi_i[15:0]按16-bit模式)，在接收第2拍(已接收32bit)时切换lane_mode_i=2'b10(8-bit)；
+2.观察rx_shift_q步进宽度从16bpc变为8bpc，数据错位；
+3.检查后续opcode_latched_q是否可能变为非法值；
+4.检查是否触发STS_BAD_OPCODE(0x02)或STS_FRAME_ERR(0x01)；
+5.模块复位后验证恢复正常工作；
+期望结果：
+1.lane_mode_i切换后bpc立即变化，rx_shift_q数据错位；
+2.错位后opcode可能为非法值→STS_BAD_OPCODE(0x02)，或rx_count失配→STS_FRAME_ERR(0x01)；
+3.模块不检测此违规，错误结果由后续命令错误暴露；
+4.复位后模块恢复正常，新事务可正常执行；
+5.验证约束：lane_mode_i在pcs_n_i=0期间必须保持稳定；
+coverage check点：
+覆盖lane_mode动态切换导致的错误场景</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TC_026</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>test_status_last_err</t>
+        </is>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+输入激励：
+1.发送正常WR_CSR命令(opcode=0x10, reg_addr=0x04, wdata=0x01)，成功后RD_CSR(STATUS=0x08)检查BUSY=0,RESP_VALID=1；
+2.发送非法opcode(0xFF)触发错误，RD_CSR(LAST_ERR=0x0C)检查ERR_CODE=0x02(BAD_OPCODE)；
+3.再发送正常RD_CSR命令(opcode=0x11, reg_addr=0x00)成功，RD_CSR(LAST_ERR)验证错误码仍为0x02(sticky)；
+4.发送另一个错误命令(bad_reg, reg_addr=0x40)，RD_CSR(LAST_ERR)验证更新为0x10(BAD_REG)；
+5.复位后RD_CSR(LAST_ERR)验证清零；
+期望结果：
+1.成功命令后STATUS.BUSY=0, STATUS.RESP_VALID=1；
+2.BAD_OPCODE后LAST_ERR=0x02，STATUS.CMD_ERR=1(sticky)；
+3.后续成功命令不影响LAST_ERR(sticky保持0x02)；
+4.BAD_REG后LAST_ERR更新为0x10；
+5.复位后LAST_ERR=0x00，STATUS所有sticky位清零；
+coverage check点：
+对STATUS各位域和LAST_ERR sticky属性收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TC_027</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>test_error_priority_chain</t>
+        </is>
+      </c>
+      <c r="C29" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，lane_mode_i=2'b11(16-bit模式)；
+2.需构造多错误同时触发的场景；
+输入激励：
+1.设置test_mode_i=0且en_i=0，发送WR_CSR(opcode=0x10, reg_addr=0x40, wdata=0x01)，同时触发NOT_IN_TEST+DISABLED+BAD_REG，验证返回STS_NOT_IN_TEST(0x04)（最高优先级）；
+2.设置test_mode_i=1且en_i=0，发送AHB_RD32(opcode=0x21, addr未对齐)，同时触发DISABLED+ALIGN_ERR，验证返回STS_DISABLED(0x08)；
+3.设置test_mode_i=1且en_i=1，发送AHB_RD_BURST(opcode=0x23, burst_len=5, addr未对齐)，同时触发ALIGN_ERR+BAD_BURST，验证返回STS_ALIGN_ERR(0x20)；
+4.设置test_mode_i=1且en_i=1，发送AHB_RD_BURST(opcode=0x23, burst_len=5, addr跨1KB)，同时触发BAD_BURST+BURST_BOUND，验证返回STS_BAD_BURST(0x80)；
+5.每次验证不产生csr_rd_en_o/csr_wr_en_o/htrans_o脉冲；
+期望结果：
+1.多错误同时触发时仅返回最高优先级错误码；
+2.优先级链：FRAME_ERR(0x01)&gt;BAD_OPCODE(0x02)&gt;NOT_IN_TEST(0x04)&gt;DISABLED(0x08)&gt;BAD_REG(0x10)&gt;ALIGN_ERR(0x20)&gt;BAD_BURST(0x80)&gt;BURST_BOUND(0x81)；
+3.所有前置错误均不发起CSR/AHB访问；
+4.STS_AHB_ERR(0x40)与前置错误互斥，仅在前置检查全部通过后可能发生；
+5.每次仅报告一个状态码，无多错误同时上报；
+coverage check点：
+对status_cp所有8个前置错误码收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC_028</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>test_align_err</t>
+        </is>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+输入激励：
+1.发送AHB_WR32(opcode=0x20, addr=0x20000001, addr[1:0]=2'b01)，验证非对齐地址检测；
+2.发送AHB_RD32(opcode=0x21, addr=0x20000002, addr[1:0]=2'b10)，验证另一种非对齐；
+3.发送AHB_RD32(opcode=0x21, addr=0x20000003, addr[1:0]=2'b11)，验证第三种非对齐；
+4.发送AHB_RD_BURST(opcode=0x23, burst_len=4, addr=0x20000001)，验证Burst非对齐检测；
+5.发送AHB_WR32(opcode=0x20, addr=0x20000000, addr[1:0]=2'b00)，验证对齐地址正常通过；
+期望结果：
+1.addr[1:0]=2'b01：返回STS_ALIGN_ERR(0x20)，htrans_o保持IDLE，不发起AHB访问；
+2.addr[1:0]=2'b10/2'b11：同样返回STS_ALIGN_ERR(0x20)；
+3.Burst非对齐：同样返回STS_ALIGN_ERR(0x20)；
+4.对齐地址(addr[1:0]=2'b00)：正常执行返回STS_OK(0x00)；
+5.ALIGN_ERR(0x20)优先级低于BAD_REG(0x10)但高于BAD_BURST(0x80)；
+coverage check点：
+覆盖addr[1:0]所有4种取值的交叉覆盖率</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC_029</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>test_frame_abort</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+输入激励：
+1.发送WR_CSR命令(opcode=0x10+reg_addr=0x04+wdata)的48-bit帧，在第3拍(已接收32bit&lt;48bit)提前拉高pcs_n_i；
+2.验证frame_abort信号产生（延迟1 cycle），返回STS_FRAME_ERR(0x01)；
+3.复位模块，发送WR_CSR命令但仅接收4bit(不足8bit，opcode未锁存)后拉高pcs_n_i；
+4.验证不产生frame_abort，接收状态静默复位；
+5.发送AHB_WR_BURST命令，在Payload接收中途拉高pcs_n_i，验证RXFIFO drain；
+期望结果：
+1.Opcode已锁存后提前终止：frame_abort=1，返回STS_FRAME_ERR(0x01)，RXFIFO drain；
+2.Opcode未锁存(接收&lt;8bit)提前终止：不产生frame_abort，不返回状态码，静默复位；
+3.Burst Payload中途终止：返回STS_FRAME_ERR(0x01)，已推入RXFIFO的数据被drain，不发起AHB Burst；
+4.FRAME_ERR(0x01)为最高优先级错误；
+5.前端FSM走IDLE→TA→TX(internal)错误返回路径，参考LRS §4.8.12；
+coverage check点：
+对帧中止时机(opcode已锁存/未锁存/Payload中途)收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC_030</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_err_response</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave配置为返回错误响应(hresp_i=1)；
+输入激励：
+1.发送AHB_RD32命令(opcode=0x21, addr=0x20000000)，AHB slave在数据相返回hresp_i=1；
+2.观察axi_state: AXI_REQ→AXI_WAIT→AXI_ERR→AXI_IDLE跳转；
+3.验证exec_status=STS_AHB_ERR(0x40), err_o=1；
+4.验证AXI_ERR下一拍自动恢复AXI_IDLE，AHB输出恢复空闲(htrans=IDLE, haddr=0)；
+5.复位后发送正常AHB_RD32命令验证模块恢复正常；
+期望结果：
+1.hresp_i=1时axi_state跳转AXI_ERR(3'b101)；
+2.返回STS_AHB_ERR(0x40)，不区分hresp错误与超时；
+3.AXI_ERR下一拍自动转AXI_IDLE(3'b000)，可立即接受新请求；
+4.AHB输出恢复空闲值；
+5.复位后新命令正常执行；
+coverage check点：
+覆盖axi_fsm_cp: AXI_ERR bin, status_cp: ahb_err bin</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC_031</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_timeout</t>
+        </is>
+      </c>
+      <c r="C33" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave配置为不响应(hready_i持续为0, hresp_i=0)；
+输入激励：
+1.发送AHB_RD32命令(opcode=0x21, addr=0x20000000)；
+2.观察timeout_cnt_q从0开始递增(每拍+1)；
+3.当timeout_cnt_q达到BUS_TIMEOUT_CYCLES-1=255时，验证触发超时；
+4.验证axi_state跳转AXI_ERR，err_o=1, exec_status=STS_AHB_ERR(0x40)；
+5.验证AXI_ERR下一拍自动恢复AXI_IDLE；
+期望结果：
+1.timeout_cnt_q在AXI_WAIT态每拍递增，AXI_REQ态清零；
+2.timeout_cnt_q==255时触发超时，跳转AXI_ERR；
+3.返回STS_AHB_ERR(0x40)，与hresp错误使用同一状态码；
+4.AXI_ERR下一拍自动转AXI_IDLE；
+5.参考LRS §4.8.13时序；
+coverage check点：
+覆盖axi_fsm_cp: AXI_WAIT(超时场景) bin</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC_032</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>test_bad_burst_len</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+输入激励：
+1.发送AHB_RD_BURST命令(opcode=0x23, burst_len=2, addr=0x20000000)，验证非法burst_len检测；
+2.发送AHB_WR_BURST命令(opcode=0x22, burst_len=3, addr=0x20000000)，验证另一种非法值；
+3.发送AHB_RD_BURST命令(opcode=0x23, burst_len=5, addr=0x20000000)；
+4.发送AHB_RD_BURST命令(opcode=0x23, burst_len=7, addr=0x20000000)；
+5.发送AHB_RD_BURST命令(opcode=0x23, burst_len=1, addr=0x20000000)，验证burst_len=1退化为Single（合法）；
+期望结果：
+1.burst_len=2：返回STS_BAD_BURST(0x80)，不发起任何AHB访问，htrans_o保持IDLE；
+2.burst_len=3/5/7：同样返回STS_BAD_BURST(0x80)；
+3.burst_len=1：退化为SINGLE等价AHB_RD32，返回STS_OK(0x00)；
+4.BAD_BURST(0x80)在优先级链中位于ALIGN_ERR(0x20)之后，与AHB_ERR(0x40)互斥；
+5.BAD_BURST仅对opcode=0x22/0x23有效；
+coverage check点：
+覆盖burst_len_cp: illegal bin, status_cp: bad_burst bin</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC_033</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>test_burst_bound</t>
+        </is>
+      </c>
+      <c r="C35" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+输入激励：
+1.发送AHB_RD_BURST×4命令(opcode=0x23, burst_len=4, addr=0x200003FC)，addr[9:0]=0x3FC+4×3=0x408≥0x400(1KB边界)，验证跨1KB边界检测；
+2.发送AHB_RD_BURST×4命令(opcode=0x23, burst_len=4, addr=0x200003F0)，addr[9:0]=0x3F0+4×3=0x3FC&lt;0x400，验证不跨边界(合法)；
+3.发送AHB_RD_BURST×8命令(opcode=0x23, burst_len=8, addr=0x200003E0)，addr[9:0]=0x3E0+4×7=0x3FC&lt;0x400(边界情况)；
+4.发送AHB_WR_BURST×16命令(opcode=0x22, burst_len=16, addr=0x20000000)，验证合法大Burst不越界；
+5.发送AHB_RD_BURST×16命令(opcode=0x23, burst_len=16, addr=0x20000FC0)，addr[9:0]=0xFC0+4×15=0x1000≥0x400，验证大Burst越界；
+期望结果：
+1.跨1KB边界：返回STS_BURST_BOUND(0x81)，不发起任何AHB访问；
+2.不跨边界：正常执行返回STS_OK(0x00)；
+3.BURST_BOUND(0x81)在优先级链中为最低优先级，位于BAD_BURST(0x80)之后；
+4.判定条件：addr[9:0]+4·(burst_len-1)&gt;=1024则为违规；
+5.该检查由SLC_DPCHK在前置阶段完成，不发起AHB事务；
+coverage check点：
+覆盖addr与1KB边界的交叉场景，status_cp: burst_bound bin</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC_034</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>test_burst_mid_error</t>
+        </is>
+      </c>
+      <c r="C36" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave配置为：前2 beat正常(hready_i=1, hresp_i=0)，第3 beat返回hresp_i=1；
+输入激励：
+1.发送AHB_RD_BURST×8命令(opcode=0x23, burst_len=8, addr=0x20000000)；
+2.观察前2 beat正常完成，hrdata_i=D0/D1推入TXFIFO(txfifo_cnt增至2)；
+3.第3 beat数据相hresp_i=1, hready_i=0（错误响应第1 cycle）；
+4.验证axi_state跳转AXI_ERR，剩余5 beat全部取消；
+5.验证第3 beat的X(invalid)数据不推入TXFIFO，TXFIFO中已有D0/D1仍发往前端；
+期望结果：
+1.前2 beat hrdata推入TXFIFO，txfifo_count_q=2；
+2.hresp_i=1后axi_state跳转AXI_ERR(3'b101)；
+3.剩余beat不再发起，htrans_o跳转IDLE；
+4.exec_status=STS_AHB_ERR(0x40)；
+5.TXFIFO中已有D0/D1仍按正常路径发往前端，ATE收到2拍而非8拍响应，参考LRS §4.8.14；
+coverage check点：
+覆盖burst中途错误场景，axi_fsm_cp: AXI_ERR bin</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TC_035</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>test_idle_toggle_suppress</t>
+        </is>
+      </c>
+      <c r="C37" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.pcs_n_i=1（空闲态）；
+输入激励：
+1.保持空闲状态100个clk_i周期，观察rx_shift_q是否不更新；
+2.观察tx_shift_q是否不翻转（非TX/TA态）；
+3.观察timeout_cnt_q是否为0（非AXI_WAIT态）；
+4.设置test_mode_i=0，观察AHB输出是否保持空闲(htrans=IDLE, hburst=SINGLE, haddr=0)；
+5.恢复test_mode_i=1，执行1次WR_CSR命令，验证模块功能正常；
+期望结果：
+1.空闲100周期内rx_shift_q值不变（门控条件：pcs_n_i=1）；
+2.tx_shift_q不翻转（门控条件：非TX/TA态）；
+3.timeout_cnt_q=0（门控条件：state!=AXI_WAIT）；
+4.test_mode_i=0时AHB输出保持空闲值；
+5.恢复后WR_CSR命令正常执行返回STS_OK(0x00)；
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>TC_009</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>test_4bit_lane</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>验证4-bit lane模式下数据收发正确性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b01(4-bit模式)；
+      <c r="D37" s="13" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TC_036</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>test_fifo_cg_behavior</t>
+        </is>
+      </c>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave正常响应(hready_i=1, hresp_i=0)；
 输入激励：
-1.通过pdi_i[3:0]按MSB-first高nibble优先发送WR_CSR帧(opcode=0x10, reg_addr=0x04, wdata=0x00000001)，共48bit=12拍；
-2.验证pdi_i[15:4]在4-bit模式下被忽略；
-3.观察turnaround 1 cycle后响应发送8bit=2拍通过pdo_o[3:0]输出；
-4.发送RD_CSR命令(opcode=0x11, reg_addr=0x04)，观察16bit RX=4拍，40bit TX=10拍；
+1.发送AHB_WR_BURST×16命令(opcode=0x22, burst_len=16, addr=0x20000000)，Payload 16×32bit=32拍RX推入RXFIFO；
+2.观察rxfifo_full_o是否在cnt达到32时拉高；
+3.RXFIFO满期间SLC_CAXIS暂停rx_shift_en和rxfifo_wr_en；
+4.后端BURST_LOOP通过rxfifo_rd_en消费，rxfifo_cnt在31/32间震荡；
+5.rxfifo_full_o清零后SLC_CAXIS恢复接收；
 期望结果：
-1.12拍RX完成，返回STS_OK(0x00)；
-2.pdo_o[3:0]输出status，pdo_o[15:4]=0；
-3.RD_CSR读回数据正确；
-4.总耗时约17 cycles（参考LRS §4.8.11）；
+1.rxfifo_count_q[5:0]增至32时rxfifo_full_o=1；
+2.RXFIFO满期间rx_shift_en=0, rxfifo_wr_en=0（门控生效）；
+3.后端消费后rxfifo_full_o清零，接收恢复；
+4.hburst_o[2:0]在整个Burst期间保持INCR16(3'b111)稳定；
+5.参考LRS §4.8.15时序；
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
-      <c r="D11" s="13" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TC_010</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>test_8bit_lane</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>验证8-bit lane模式下数据收发正确性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b10(8-bit模式)；
+      <c r="D38" s="13" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TC_037</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>test_wr_burst16_throughput</t>
+        </is>
+      </c>
+      <c r="C39" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave zero-wait-state(hready_i=1, hresp_i=0)；
 输入激励：
-1.通过pdi_i[7:0]按MSB-first发送WR_CSR帧(opcode=0x10, reg_addr=0x04, wdata=0x00000005)，共48bit=6拍；
-2.验证pdi_i[15:8]在8-bit模式下被忽略；
-3.观察响应发送8bit=1拍通过pdo_o[7:0]输出；
-4.发送AHB_RD32命令(opcode=0x21, addr=0x10000000)，观察40bit RX=5拍，40bit TX=5拍；
+1.发送AHB_WR_BURST×16命令(opcode=0x22, burst_len=16, addr=0x20000000, wdata×16随机数据)；
+2.测量端到端延时（从pcs_n_i拉低到pdo_oe_o拉高释放完成）；
+3.计算有效吞吐：64B payload / 总cycles × 100MHz；
+4.重复执行5次取平均；
+5.验证hburst_o=INCR16(3'b111), hsize_o=3'b010(WORD), haddr每拍+4；
 期望结果：
-1.6拍RX完成，返回STS_OK(0x00)；
-2.pdo_o[7:0]输出status，pdo_o[15:8]=0；
-3.AHB_RD32命令正常完成，读回hrdata正确；
+1.端到端延时约54~56 cycles/64B；
+2.有效写吞吐约116MB/s；
+3.hburst_o=INCR16(3'b111)在整个burst期间稳定；
+4.NONSEQ+SEQ×15地址相完整，hwdata_o 16拍数据正确；
+5.status_code=STS_OK(0x00)；
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TC_011</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>test_16bit_lane</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>验证16-bit lane模式下数据收发正确性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
+      <c r="D39" s="13" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>TC_038</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>test_rd_burst16_throughput</t>
+        </is>
+      </c>
+      <c r="C40" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave zero-wait-state(hready_i=1, hresp_i=0, hrdata_i递增数据)；
 输入激励：
-1.通过pdi_i[15:0]按MSB-first发送WR_CSR帧(opcode=0x10, reg_addr=0x04, wdata=0x0000000F)，共48bit=3拍；
-2.验证pdi_i[15:0]全部有效，无忽略位；
-3.观察响应发送8bit=1拍通过pdo_o[15:0]输出（status+8bit padding）；
-4.依次发送AHB_WR32(opcode=0x20)、AHB_RD32(opcode=0x21)命令验证16-bit模式全流程；
+1.发送AHB_RD_BURST×16命令(opcode=0x23, burst_len=16, addr=0x20000000)；
+2.测量端到端延时（从pcs_n_i拉低到TX完成）；
+3.计算有效吞吐：64B payload / 总cycles × 100MHz；
+4.验证hburst_o=INCR16(3'b111), htrans_o: NONSEQ+SEQ×15, haddr: A/A+4/.../A+0x3C；
+5.验证33拍TX输出status(8bit)+rdata×16(512bit)=520bit；
 期望结果：
-1.3拍RX完成，返回STS_OK(0x00)；
-2.pdo_o[15:0]输出status+padding，MSB-first；
-3.AHB_WR32/AHB_RD32正常完成，有效吞吐约200MB/s原始线速；
+1.端到端延时约54 cycles/64B；
+2.有效读吞吐约118MB/s；
+3.hburst_o=INCR16(3'b111)稳定，17拍AHB执行(NONSEQ+SEQ×15+末beat数据相)；
+4.16个beat hrdata_i全部正确采样并推入TXFIFO；
+5.status_code=STS_OK(0x00)；
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
-      <c r="D13" s="13" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TC_012</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>test_wr_csr_data_interface</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>验证WR_CSR命令在16-bit模式下帧接收、CSR接口和响应时序的正确性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)，pcs_n_i初始为高电平；
+      <c r="D40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>TC_039</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>test_dfx_counters</t>
+        </is>
+      </c>
+      <c r="C41" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave正常响应；
 输入激励：
-1.ATE拉低pcs_n_i开始帧传输，按MSB-first顺序通过pdi_i[15:0]发送WR_CSR帧(opcode=0x10+reg_addr=0x04+wdata=0x00000001)；
-2.观察3拍RX(48bit)完成后frame_valid延迟1 cycle拉高；
-3.观察csr_wr_en_o产生1周期脉冲，同周期csr_addr_o=0x04，csr_wdata_o=0x01；
-4.观察1 cycle turnaround后pdo_oe_o拉高，模块驱动pdo_o[15:0]输出响应；
-5.1拍TX输出status byte后pdo_oe_o释放，pcs_n_i拉高；
+1.执行3次WR_CSR(opcode=0x10)成功命令，读取WR_CSR成功计数器验证值为3；
+2.执行2次非法opcode(0xFF)失败命令，读取BAD_OPCODE(0x02)失败计数器验证值为2；
+3.执行1次AHB_RD_BURST×4(opcode=0x23)成功，读取INCR4读成功计数器验证值为1；
+4.对WR_CSR成功计数器执行WC写1清零，验证计数器归零；
+5.读取CSR读/写计数器、AHB Single读/写计数器验证正确性；
 期望结果：
-1.frame_valid延迟1 cycle拉高，front_state: IDLE→ISSUE→WAIT_RESP→TA→TX→IDLE；
-2.csr_wr_en_o单周期脉冲，csr_addr_o=0x04(CTRL)，csr_wdata_o=0x00000001；
-3.turnaround 1 cycle后pdo_oe_o=1，1拍TX输出STS_OK(0x00)；
-4.pdo_oe_o释放后pcs_n_i拉高，回到IDLE；
+1.WR_CSR成功计数器=3，WC写1后归零；
+2.BAD_OPCODE失败计数器=2；
+3.INCR4读成功计数器=1；
+4.CSR写计数器≥3(CSR write次数), CSR读计数器≥计数器读取次数；
+5.所有计数器位宽≥16bit，短期不溢出；
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
-      <c r="D14" s="13" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>TC_013</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>test_4bit_wr_csr</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>验证4-bit模式下WR_CSR命令帧接收和响应发送的完整时序。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b01(4-bit模式)；
+      <c r="D41" s="13" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>TC_040</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>test_dfx_fsm_observability</t>
+        </is>
+      </c>
+      <c r="C42" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave正常响应；
 输入激励：
-1.ATE拉低pcs_n_i，通过pdi_i[3:0]发送WR_CSR帧(opcode=0x10+reg_addr=0x04+wdata=0x00000003)，12拍RX(48bit/4bpc)；
-2.观察接收12拍完成后frame_valid脉冲；
-3.观察1 cycle turnaround后pdo_oe_o拉高；
-4.观察响应发送2拍(8bit/4bpc)输出status byte；
-5.pdo_oe_o释放，pcs_n_i拉高结束事务；
+1.发送WR_CSR命令期间观察front_state_q[2:0]变化：IDLE(3'd0)→ISSUE(3'd1)→WAIT_RESP(3'd2)→TA(3'd3)→TX(3'd4)→IDLE；
+2.发送AHB_RD32命令期间观察axi_state_q[2:0]变化：AXI_IDLE→AXI_REQ→AXI_WAIT→AXI_DONE→AXI_IDLE；
+3.发送AHB_WR_BURST×4命令期间观察back_state_q[2:0]变化：S_IDLE→S_LOAD_TASK→S_EXEC→S_BURST_LOOP→S_BUILD_RESP→S_DONE→S_IDLE；
+4.在Burst执行期间读取rxfifo_count_q[5:0]/txfifo_count_q[5:0]验证FIFO占用；
+5.验证burst_beat_cnt_q[4:0]在BURST_LOOP期间从0递增至burst_len-1；
 期望结果：
-1.12拍RX完成，frame_valid延迟1 cycle；
-2.turnaround 1 cycle，pdo_oe_o在TX期间=1；
-3.2拍TX输出STS_OK(0x00)；
-4.总耗时约17 cycles（参考LRS §4.8.11）；
+1.front_state_q完整经历6态；
+2.axi_state_q完整经历6态(不含AXI_BURST因Single无burst)；
+3.back_state_q完整经历7态(含S_BURST_LOOP)；
+4.rxfifo_count_q/txfifo_count_q正确反映FIFO占用；
+5.burst_beat_cnt_q从0递增，参考LRS §10.2；
+coverage check点：
+对front_fsm_cp/back_fsm_cp/axi_fsm_cp所有状态收集功能覆盖率</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>TC_041</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>test_memmap_access</t>
+        </is>
+      </c>
+      <c r="C43" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave正常响应(hready_i=1, hresp_i=0)；
+输入激励：
+1.通过RD_CSR(opcode=0x11, reg_addr=0x00)访问内部CSR，验证CSR不经过AHB总线(无htrans_o NONSEQ脉冲)；
+2.通过AHB_WR32(opcode=0x20, addr=0x20000000)访问外部SoC地址，验证htrans_o=NONSEQ发起AHB事务；
+3.通过AHB_RD32(opcode=0x21, addr=0x30000000)访问另一SoC地址，验证可达不同地址段；
+4.对非法SoC地址(addr导致SoC解码器返回hresp_i=1)发送AHB命令，验证返回STS_AHB_ERR(0x40)；
+5.验证CSR接口和AHB接口不会同时激活（单任务串行执行）；
+期望结果：
+1.CSR访问：csr_rd_en_o=1脉冲，htrans_o保持IDLE，CSR不进入AHB memory map；
+2.AHB访问：htrans_o=NONSEQ，haddr_o=0x20000000，发起AHB事务；
+3.不同SoC地址均可访问（模块不做无效地址判决）；
+4.SoC返回hresp_i=1时统一映射STS_AHB_ERR(0x40)；
+5.CSR和AHB访问不会并发，单任务串行；
 coverage check点：
 直接用例覆盖，不收功能覆盖率</t>
         </is>
       </c>
-      <c r="D15" s="13" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>TC_014</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>test_rd_csr_frame</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>验证RD_CSR命令在16-bit模式下请求帧和响应帧格式。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
+      <c r="D43" s="13" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>TC_042</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_rd32_protocol_detail</t>
+        </is>
+      </c>
+      <c r="C44" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave zero-wait-state(hready_i=1, hresp_i=0, hrdata_i=0xABCD1234)；
 输入激励：
-1.发送RD_CSR命令(opcode=0x11, reg_addr=0x00(VERSION))，请求帧16bit=1拍RX；
-2.观察csr_rd_en_o产生1周期脉冲，csr_addr_o=0x00；
-3.观察下一周期csr_rdata_i[31:0]由外部CSR File驱动（1 cycle读延迟）；
-4.观察1 cycle turnaround后pdo_oe_o拉高，3拍TX输出40-bit响应(status+rdata)；
-5.读取status byte验证为STS_OK(0x00)；
+1.发送AHB_RD32命令(opcode=0x21, addr=0x20000000)；
+2.详细验证AXI_REQ态：htrans_o[1:0]=2'b10(NONSEQ), haddr_o=0x20000000, hwrite_o=0, hsize_o[2:0]=3'b010, hburst_o[2:0]=3'b000(SINGLE)；
+3.详细验证AXI_WAIT态：htrans_o=2'b00(IDLE), hready_i=1时采样hrdata_i=0xABCD1234；
+4.详细验证AXI_DONE态：AHB输出释放，htrans_o保持IDLE；
+5.验证地址相(T1)和数据相(T2)错开1拍（2-phase流水）；
 期望结果：
-1.1拍RX完成，frame_valid延迟1 cycle；
-2.csr_rd_en_o单周期脉冲，下一周期csr_rdata_i有效；
-3.3拍TX输出[status(8)|VERSION(32)]，MSB-first；
-4.status_code=STS_OK(0x00)；
+1.AXI_REQ(1拍): htrans=NONSEQ + haddr + hwrite=0 + hsize=WORD + hburst=SINGLE；
+2.AXI_WAIT(1拍): htrans=IDLE, 采样hrdata=0xABCD1234；
+3.AXI_DONE(1拍): 释放AHB；
+4.地址相与数据相overlap 1拍，写操作haddr与hwdata错开1拍；
+5.参考LRS §4.8.5完整时序；
 coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D16" s="13" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>TC_015</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>test_ahb_wr32_frame</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>验证AHB_WR32命令在16-bit模式下请求帧格式和AHB事务时序。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
+覆盖axi_fsm_cp: AXI_REQ/AXI_WAIT/AXI_DONE</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>TC_043</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_incr4_protocol</t>
+        </is>
+      </c>
+      <c r="C45" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave正常响应(hready_i=1, hresp_i=0, hrdata_i按beat递增D0~D3)；
 输入激励：
-1.发送AHB_WR32命令(opcode=0x20, addr=0x10000000, wdata=0xCAFEBABE)，请求帧72bit=5拍RX；
-2.观察front_state: IDLE→ISSUE→WAIT_RESP→TA→TX→IDLE；
-3.观察axi_state: AXI_IDLE→AXI_REQ→AXI_WAIT→AXI_DONE→AXI_IDLE；
-4.观察htrans_o=NONSEQ(2'b10), haddr_o=0x10000000, hwrite_o=1, hburst_o=SINGLE(3'b000)；
-5.观察hwdata_o=0xCAFEBABE在数据相驱动，hready_i=1时完成；
-6.观察1拍TX输出STS_OK(0x00)；
+1.发送AHB_RD_BURST×4命令(opcode=0x23, burst_len=4, addr=0x20000000)；
+2.详细验证4拍地址相：htrans_o=NONSEQ→SEQ→SEQ→SEQ, haddr_o=A→A+4→A+8→A+C, hburst_o=INCR4(3'b011)保持稳定；
+3.详细验证4拍数据相：hrdata_i=D0→D1→D2→D3，地址相与数据相overlap 1拍；
+4.验证末beat数据相后htrans_o=IDLE，AXI_DONE释放AHB；
+5.验证resp_valid和resp_last时序；
 期望结果：
-1.5拍RX完成，72-bit帧正确解析；
-2.htrans_o=NONSEQ单拍, hsize_o=3'b010(WORD)；
-3.hwdata_o在地址相下一拍有效（2-phase流水）；
-4.status_code=STS_OK(0x00)；
+1.4拍地址相hburst_o[2:0]=3'b011(INCR4)全程稳定不翻转；
+2.htrans_o序列: NONSEQ(2'b10)→SEQ(2'b11)×3→IDLE(2'b00)；
+3.haddr每拍+4：A/A+4/A+8/A+0xC；
+4.hrdata_i 4拍数据全部正确采样，推入TXFIFO；
+5.参考LRS §4.8.9内部INCR4时序；
 coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>TC_016</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>test_ahb_rd32_frame</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>验证AHB_RD32命令在16-bit模式下请求帧和响应帧格式。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
+覆盖burst_len_cp: incr4 bin, axi_fsm_cp: AXI_BURST</t>
+        </is>
+      </c>
+      <c r="D45" s="13" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>TC_044</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>test_ahb_wr_burst16_protocol</t>
+        </is>
+      </c>
+      <c r="C46" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave正常响应(hready_i=1, hresp_i=0)；
 输入激励：
-1.发送AHB_RD32命令(opcode=0x21, addr=0x10000000)，请求帧40bit=3拍RX；
-2.观察axi_state: AXI_IDLE→AXI_REQ→AXI_WAIT→AXI_DONE→AXI_IDLE；
-3.观察htrans_o=NONSEQ(2'b10), hwrite_o=0, hburst_o=SINGLE(3'b000)；
-4.观察hrdata_i[31:0]在hready_i=1时被采样；
-5.观察3拍TX输出40-bit响应(status+rdata)；
+1.发送AHB_WR_BURST×16命令(opcode=0x22, burst_len=16, addr=0x20000000, wdata×16递增0~15)；
+2.验证hburst_o=INCR16(3'b111)保持稳定，htrans_o: NONSEQ→SEQ×15→IDLE，hsize_o=3'b010(WORD)；
+3.验证16拍hwdata_o依次输出wdata[0]~wdata[15]（数据相与地址相overlap 1拍）；
+4.验证后端从RXFIFO读出16个beat数据作为hwdata_o输出；
+5.验证back_state经历S_BURST_LOOP态；
 期望结果：
-1.3拍RX完成，40-bit帧正确解析；
-2.haddr_o=0x10000000, hsize_o=3'b010, hwrite_o=0；
-3.hrdata_i在hready_i=1上升沿被采样，组装进响应帧；
-4.3拍TX输出[status(8)|rdata(32)]，status_code=STS_OK(0x00)；
+1.hburst_o[2:0]=3'b111(INCR16)在整个burst期间稳定；
+2.htrans_o: NONSEQ(1拍)→SEQ(15拍)→IDLE，haddr每拍+4；
+3.hwdata_o 16拍数据正确，与RXFIFO读出顺序一致；
+4.hsize_o=3'b010(WORD)全程不变；
+5.status_code=STS_OK(0x00)；
 coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D18" s="13" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>TC_017</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>test_ahb_rd_burst4</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>验证AHB_RD_BURST×4命令端到端时序和AHB INCR4行为。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)，AHB zero-wait-state；
+覆盖burst_len_cp: incr16 bin, back_fsm_cp: S_BURST_LOOP</t>
+        </is>
+      </c>
+      <c r="D46" s="13" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>TC_045</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>test_rxfifo_backpressure</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave配置为延迟响应（每beat等待3周期hready_i=1），以制造FIFO满场景；
 输入激励：
-1.发送AHB_RD_BURST命令(opcode=0x23, burst_len=4, addr=0x10000000)，3拍RX header；
-2.观察task_req/task_ack一拍握手下发task_desc给SLC_BANK；
-3.观察AHB地址相：htrans_o=NONSEQ首拍，SEQ×3后续拍，hburst_o=INCR4(3'b011)保持稳定；
-4.观察haddr_o每拍+4：0x10000000→0x10000004→0x10000008→0x1000000C；
-5.观察hrdata_i[31:0]连续4 beat被采样推入TXFIFO；
-6.观察1 cycle turnaround后TX_BURST从TXFIFO串行发送status+4×32-bit rdata；
+1.发送AHB_WR_BURST×16命令(opcode=0x22, burst_len=16, addr=0x20000000)，Payload 32拍推入RXFIFO；
+2.观察rxfifo_count_q增至32时rxfifo_full_o=1；
+3.RXFIFO满期间SLC_CAXIS暂停rx_shift_en和rxfifo_wr_en；
+4.后端BURST_LOOP通过rxfifo_rd_en消费1 word后rxfifo_cnt降至31，rxfifo_full_o清零；
+5.恢复接收后续Payload beat，直至全部16 beat发送完成；
 期望结果：
-1.hburst_o=INCR4(3'b011)在整个burst地址相期间保持稳定；
-2.haddr_o每拍+4，地址序列正确；
-3.status_code=STS_OK(0x00) + 4 beat rdata正确；
-4.Burst读响应beat间无turnaround，pdo_oe_o连续有效；
+1.rxfifo_full_o=1期间rx_shift_en=0, rxfifo_wr_en=0（反压生效）；
+2.后端消费后rxfifo_full_o清零，接收恢复；
+3.最终所有16 beat数据正确写入AHB；
+4.rxfifo_count_q在满/未满间震荡，参考LRS §4.8.15；
+5.status_code=STS_OK(0x00)；
 coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>TC_018</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>test_ahb_rd_burst8</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>验证AHB_RD_BURST×8命令INCR8时序和响应发送。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)，AHB zero-wait-state；
+覆盖rxfifo_full反压场景</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>TC_046</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>test_txfifo_stall</t>
+        </is>
+      </c>
+      <c r="C48" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave配置为间歇延迟响应（前4 beat正常，后4 beat每beat等待5周期），以制造TXFIFO空场景；
 输入激励：
-1.发送AHB_RD_BURST命令(opcode=0x23, burst_len=8, addr=0x10000000)，3拍RX header；
-2.观察hburst_o=INCR8(3'b101)在整个burst保持稳定；
-3.观察htrans_o: NONSEQ+SEQ×7，haddr_o每拍+4共8个地址；
-4.观察8 beat hrdata连续采样；
-5.观察resp_last在末beat置位，Burst结束；
-6.观察TX_BURST发送status+8×32-bit rdata，共17拍TX(8+32×8=264bit)；
+1.发送AHB_RD_BURST×8命令(opcode=0x23, burst_len=8, addr=0x20000000)；
+2.观察前4 beat hrdata推入TXFIFO后，SLC_SAXIS开始TX_BURST发送；
+3.当TXFIFO消费快于后端写入时，txfifo_empty_o=1；
+4.验证TXFIFO空时pdo_oe_o保持高电平(不释放总线方向)，pdo_o[15:0]保持上一拍数据值；
+5.下一beat到达后立即恢复移位输出；
 期望结果：
-1.hburst_o=INCR8(3'b101)保持稳定，不逐beat切换；
-2.NONSEQ+SEQ×7地址相序列正确；
-3.status_code=STS_OK(0x00) + 8 beat rdata正确；
-4.最小端到端延时约19~21 cycles（参考LRS §5.2.1）；
+1.TX_BURST期间txfifo_empty_o=1时TX暂停，pdo_oe_o=1持续有效；
+2.pdo_o[15:0]保持上一拍数据值（非HiZ）；
+3.TXFIFO非空后立即恢复移位；
+4.Burst读响应beat间无turnaround；
+5.最终所有8 beat数据正确输出，status_code=STS_OK(0x00)，参考LRS §3.5.2；
 coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>TC_019</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>test_ahb_wr_burst4</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>验证AHB_WR_BURST×4命令端到端时序，包括RXFIFO写入和后端读取。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)，AHB zero-wait-state；
-输入激励：
-1.发送AHB_WR_BURST命令(opcode=0x22, burst_len=4, addr=0x10000000)，3拍RX header + 8拍RX payload(4×32bit)；
-2.观察rxfifo_wr_en每凑够32-bit推入SLC_RXFIFO，共4次写入(D0,D1,D2,D3)；
-3.观察front_state: IDLE→ISSUE→WAIT_RESP→TA→TX→IDLE；
-4.观察后端BURST_LOOP从RXFIFO读取数据作为hwdata_o；
-5.观察hburst_o=INCR4(3'b011)，hwrite_o=1，haddr_o每拍+4；
-6.观察1拍TX输出STS_OK(0x00)；
-期望结果：
-1.RXFIFO写入4 beat，后端读出4 beat作为hwdata_o(D0,D1,D2,D3)；
-2.hburst_o=INCR4保持稳定，hsize_o=3'b010(WORD)；
-3.hwdata_o与haddr_o错开1拍（2-phase流水）；
-4.status_code=STS_OK(0x00)；
-coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>TC_020</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>test_bad_opcode</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>验证非法opcode被前置检查拒绝并返回STS_BAD_OPCODE。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送opcode=0xFF的命令帧（非法opcode，不在0x10/0x11/0x20/0x21/0x22/0x23中）；
-2.发送opcode=0x00的命令帧；
-3.发送opcode=0x24的命令帧（紧邻合法范围上界）；
-4.发送opcode=0x0F的命令帧（紧邻合法范围下界）；
-期望结果：
-1.所有非法opcode返回STS_BAD_OPCODE(0x02)；
-2.不产生csr_rd_en_o/csr_wr_en_o/htrans_o脉冲；
-3.前端FSM走IDLE→TA→TX错误返回路径；
-4.非法opcode不发起任何CSR/AHB访问；
-coverage check点：
-对opcode空间0x00~0xFF边界收集功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>TC_021</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>test_legal_opcode_sweep</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>验证6种合法opcode均能正确解码执行并返回STS_OK。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送WR_CSR命令(opcode=0x10, reg_addr=0x04, wdata=0x01)，验证返回STS_OK；
-2.发送RD_CSR命令(opcode=0x11, reg_addr=0x04)，验证返回STS_OK+rdata；
-3.发送AHB_WR32命令(opcode=0x20, addr=0x10000000, wdata=0xDEADBEEF)，验证返回STS_OK；
-4.发送AHB_RD32命令(opcode=0x21, addr=0x10000000)，验证返回STS_OK+rdata；
-5.发送AHB_WR_BURST命令(opcode=0x22, burst_len=4, addr=0x20000000, wdata=4beat)，验证返回STS_OK；
-6.发送AHB_RD_BURST命令(opcode=0x23, burst_len=4, addr=0x20000000)，验证返回STS_OK+4 beat rdata；
-期望结果：
-1.所有6种opcode正确解码执行，每条返回STS_OK(0x00)；
-2.CSR命令产生csr_wr_en_o/csr_rd_en_o脉冲，AHB命令产生htrans_o=NONSEQ；
-3.每条命令执行后模块回到IDLE态，可立即接受下一条命令；
-4.Burst命令hburst_o正确映射：burst_len=4→INCR4(3'b011)；
-coverage check点：
-覆盖所有6种opcode的译码和执行路径</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>TC_022</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>test_lane_switch_idle</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>验证空闲态下lane_mode切换成功，新事务按新模式执行。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.pcs_n_i=1（空闲态），初始lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.在16-bit模式下发送WR_CSR命令(opcode=0x10, reg_addr=0x04, wdata=0x01)，3拍RX，验证正常执行；
-2.命令结束后（pcs_n_i=1），切换lane_mode_i从2'b11→2'b00(1-bit模式)；
-3.等待2个clk_i周期同步；
-4.在1-bit模式下发送RD_CSR命令(opcode=0x11, reg_addr=0x04)，16拍RX(16bit/1bpc)，验证正常执行；
-5.再切换lane_mode_i从2'b00→2'b01(4-bit模式)，等待2周期后发送命令验证；
-期望结果：
-1.16-bit命令正常执行，3拍RX完成；
-2.切换至1-bit后，16拍RX完成，接收拍数正确增加；
-3.切换至4-bit后，4拍RX完成，接收拍数正确；
-4.每次切换后命令返回STS_OK(0x00)，数据正确；
-coverage check点：
-对lane_mode切换场景(16→1, 1→4)收集功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>TC_023</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>test_lane_switch_during_tx</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>验证事务执行期间切换lane_mode_i导致帧数据错位和错误行为。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)，pcs_n_i=0（事务进行中）；
-输入激励：
-1.拉低pcs_n_i开始WR_CSR事务，按16-bit模式发送前2拍(opcode+reg_addr已发送)；
-2.在RX阶段第3拍前切换lane_mode_i从2'b11→2'b10(8-bit模式)（违反约束！）；
-3.继续发送数据，观察模块后续行为；
-4.等待事务结束，检查status_code；
-期望结果：
-1.lane_mode切换后移位寄存器步进宽度bpc立即从16变为8，帧数据错位；
-2.可能误触发STS_BAD_OPCODE(0x02)或STS_FRAME_ERR(0x01)；
-3.模块不检测此违规行为，由集成方保证lane_mode_i稳定性；
-4.接收数据损坏，rx_shift_q内容不可预测；
-coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>TC_024</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>test_status_polling</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>验证STATUS/LAST_ERR寄存器状态报告正确性，包括sticky行为验证。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.执行正常WR_CSR命令后，读取STATUS(opcode=0x11, reg_addr=0x08)，记录STATUS值；
-2.执行错误命令（RD_CSR, reg_addr=0x40触发STS_BAD_REG），读取STATUS和LAST_ERR(opcode=0x11, reg_addr=0x0C)；
-3.在错误之后执行一条正常命令（WR_CSR, reg_addr=0x04），再次读取LAST_ERR，验证sticky——错误码仍存在；
-4.执行Burst命令后读取STATUS，验证BURST_ERR位；
-5.确认无独立中断输出端口，仅能通过轮询STATUS/LAST_ERR获取状态；
-期望结果：
-1.正常命令后STATUS.BUSY=0，RESP_VALID=1；
-2.错误命令后STATUS.CMD_ERR=1(sticky)，LAST_ERR保存错误码0x10；
-3.中间插入正常命令后LAST_ERR仍为0x10，证明sticky属性——错误码不会被后续成功命令覆盖；
-4.无中断输出信号，状态仅通过寄存器查询获取；
-coverage check点：
-对STATUS各bit位和LAST_ERR sticky行为收集功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>TC_025</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>test_frame_abort</t>
-        </is>
-      </c>
-      <c r="C27" s="21" t="inlineStr">
-        <is>
-          <t>验证帧中止(pcs_n_i提前释放)在不同时机的行为，包括opcode已锁存和未锁存两种场景。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)，pcs_n_i初始为高电平；
-输入激励：
-1.正常帧传输：ATE拉低pcs_n_i开始帧传输，按MSB-first顺序通过pdi_i[15:0]发送RD_CSR帧(opcode=0x11+reg_addr=0x00)；
-2.等待1个turnaround周期，检查pdo_oe_o拉高，模块驱动pdo_o[15:0]输出响应；
-3.帧中止场景1：发送WR_CSR命令(opcode=0x10+reg_addr=0x04+wdata=0x01)但在接收16bit后(已锁存opcode)提前拉高pcs_n_i；
-4.复位模块，帧中止场景2：发送RD_CSR命令但在接收4bit后(opcode未锁存，接收&lt;8bit)提前拉高pcs_n_i；
-期望结果：
-1.正常帧：pcs_n_i=0期间接收数据，turnaround后pdo_oe_o=1驱动响应，status_code=STS_OK(0x00)；
-2.帧中止场景1(opcode已锁存)：返回STS_FRAME_ERR(0x01)，pdo_oe_o拉高后输出状态码；
-3.帧中止场景2(opcode未锁存)：接收状态静默复位，不产生frame_abort，不输出响应帧；
-coverage check点：
-对帧中止时机(opcode已锁存/未锁存)收集功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>TC_026</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>test_ahb_timeout</t>
-        </is>
-      </c>
-      <c r="C28" s="21" t="inlineStr">
-        <is>
-          <t>验证AHB超时检测和错误返回机制。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送AHB_RD32命令(opcode=0x21, addr=0x10000000)；
-2.Force hready_i=0持续257个clk_i周期（超过BUS_TIMEOUT_CYCLES=256）；
-3.观察timeout_cnt[8:0]从0递增至255的过程；
-4.当timeout_cnt=255时观察axi_state跳转AXI_ERR，err_o=1；
-5.观察AXI_ERR→AXI_IDLE自动恢复；
-6.恢复后发送新命令验证模块可正常工作；
-期望结果：
-1.timeout_cnt从0递增至255(BUS_TIMEOUT_CYCLES-1)，每AXI_WAIT拍+1；
-2.axi_state跳转AXI_ERR，返回STS_AHB_ERR(0x40)；
-3.AXI_ERR下一拍自动恢复至AXI_IDLE；
-4.AHB输出恢复空闲：htrans_o=IDLE，hburst_o=SINGLE，haddr_o=0x0；
-5.恢复后新命令正常执行，status_code=STS_OK(0x00)；
-coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>TC_027</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>test_rxfifo_backpressure</t>
-        </is>
-      </c>
-      <c r="C29" s="21" t="inlineStr">
-        <is>
-          <t>验证RXFIFO满反压机制：SLC_CAXIS暂停接收，后端消费后恢复。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送AHB_WR_BURST×16命令(opcode=0x22, burst_len=16, addr=0x10000000)，填充16 beat payload；
-2.控制后端慢消费（延迟rxfifo_rd_en），使rxfifo_cnt[5:0]增至32；
-3.观察rxfifo_full_o=1时SLC_CAXIS行为：rx_shift_en=0，rxfifo_wr_en=0暂停接收；
-4.后端开始消费（rxfifo_rd_en拉高），rxfifo_cnt降至31后rxfifo_full_o=0；
-5.SLC_CAXIS恢复接收后续payload beat；
-期望结果：
-1.rxfifo_cnt增至32时rxfifo_full_o=1，接收暂停；
-2.rxfifo_full_o=1期间rx_shift_en=0，rxfifo_wr_en=0；
-3.后端drain后rxfifo_full_o=0，恢复接收；
-4.最终16 beat全部正确写入AHB，status_code=STS_OK(0x00)；
-coverage check点：
-对rxfifo_cnt边界值(31,32)和rxfifo_full_o跳变收集功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D29" s="13" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>TC_028</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>test_txfifo_stall</t>
-        </is>
-      </c>
-      <c r="C30" s="21" t="inlineStr">
-        <is>
-          <t>验证TXFIFO空时TX暂停行为：pdo_oe_o保持高，等待下一beat到达后恢复。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.执行AHB_RD_BURST×16命令(opcode=0x23, burst_len=16, addr=0x10000000)；
-2.在TX_BURST阶段制造后端延迟（控制txfifo_wr_en），使txfifo_empty_o=1出现；
-3.观察txfifo_empty_o=1时SLC_SAXIS行为：pdo_oe_o保持高电平不释放；
-4.观察pdo_o[15:0]保持上一拍数据值（非HiZ）；
-5.当下一beat到达TXFIFO后，观察SLC_SAXIS立即恢复移位输出；
-期望结果：
-1.txfifo_empty_o=1时pdo_oe_o保持1（不主动释放总线方向）；
-2.pdo_o[15:0]保持上一拍数据值，不出现HiZ或无效数据；
-3.下一beat到达后立即恢复移位，无额外延迟；
-4.Burst响应beat间无turnaround，pdo_oe_o连续有效；
-coverage check点：
-直接用例覆盖，不收功能覆盖率</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>TC_029</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_config_sweep</t>
-        </is>
-      </c>
-      <c r="C31" s="21" t="inlineStr">
-        <is>
-          <t>随机配置遍历：遍历所有有效lane_mode×opcode×burst_len组合。
-配置条件：
+覆盖txfifo_empty反压场景</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>TC_047</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>test_rand_csr_access</t>
+        </is>
+      </c>
+      <c r="C49" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
 1.模块复位完成，test_mode_i=1，en_i=1；
 2.随机配置lane_mode_i[1:0]（遍历2'b00/01/10/11）；
 输入激励：
-1.随机选择lane_mode_i（遍历4种模式）；
-2.随机选择opcode（遍历0x10/0x11/0x20/0x21/0x22/0x23）；
-3.对于Burst命令，随机选择burst_len（遍历1/4/8/16）；
-4.随机生成地址（addr需4-byte对齐，addr[1:0]=2'b00）；
-5.对于写命令，随机生成wdata；
-6.重复执行N次（N≥100），每次随机配置；
-7.验证每条命令响应status_code正确；
+1.随机选择opcode（遍历0x10/0x11 WR_CSR/RD_CSR）；
+2.随机选择reg_addr（遍历0x00/0x04/0x08/0x0C/0x10合法地址和0x40/0xFF非法地址）；
+3.随机生成wdata（32-bit随机值）；
+4.重复执行N次（N≥100），每次随机配置lane_mode和参数；
+5.对非法地址验证返回STS_BAD_REG(0x10)，对合法地址验证STS_OK(0x00)；
+6.对所有RW寄存器验证写入后读回一致，对RO寄存器验证写入无效；
 期望结果：
-1.成功场景：status_code=STS_OK(0x00)；
-2.所有配置组合均被覆盖；
-3.各lane_mode下帧接收拍数正确：RX拍数=帧长/bpc；
-4.Burst命令hburst_o正确映射；
+1.成功场景：合法CSR访问返回STS_OK(0x00)，RW属性正确，RO属性正确；
+2.失败场景：非法地址返回STS_BAD_REG(0x10)；
+3.所有lane_mode下CSR访问功能一致；
+4.WC寄存器写1清零，写0不清零；
 coverage check点：
 1.覆盖lane_mode所有取值：2'b00, 2'b01, 2'b10, 2'b11；
-2.覆盖所有opcode：0x10, 0x11, 0x20, 0x21, 0x22, 0x23；
-3.覆盖所有burst_len：1, 4, 8, 16；
-4.覆盖lane_mode × opcode所有组合</t>
-        </is>
-      </c>
-      <c r="D31" s="13" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>TC_030</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_data_payload</t>
-        </is>
-      </c>
-      <c r="C32" s="21" t="inlineStr">
-        <is>
-          <t>随机数据payload测试：随机wdata/rdata和随机对齐地址。
-配置条件：
+2.覆盖reg_addr边界值：0x00, 0x04, 0x08, 0x0C, 0x10, 0x3F(合法), 0x40(非法)；
+3.覆盖lane_mode × opcode(WR_CSR/RD_CSR)所有组合</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>TC_048</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>test_rand_lane_opcode</t>
+        </is>
+      </c>
+      <c r="C50" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
 1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
+2.使用嵌套循环遍历所有组合；
 输入激励：
-1.随机选择命令类型（AHB_WR32/AHB_RD32/AHB_WR_BURST/AHB_RD_BURST）；
-2.随机生成4-byte对齐地址（addr[1:0]=2'b00）；
-3.对于写命令，随机生成wdata[31:0]（含全0、全1、0xAAAAAAAA等特殊值）；
-4.对于Burst命令，随机选择burst_len∈{4,8,16}，每个beat随机wdata；
-5.执行写后读回验证数据一致性；
-6.重复执行N次（N≥200），每次随机数据；
+1.for lane_mode in [2'b00, 2'b01, 2'b10, 2'b11]: 随机选择opcode（遍历0x10/0x11/0x20/0x21/0x22/0x23）；
+2.对于Burst命令，随机选择burst_len（遍历1/4/8/16）；
+3.随机生成地址（addr需4-byte对齐）和wdata；
+4.每次配置后等待≥2周期同步，然后拉低pcs_n_i发送命令；
+5.重复执行N次（N≥100），每次随机组合lane_mode和opcode；
 期望结果：
-1.所有命令返回STS_OK(0x00)；
-2.写后读回数据一致，hwdata_o=写入值；
-3.Burst写每个beat数据正确到达AHB slave；
-4.特殊数据值（全0/全1/交替）无异常；
+1.所有lane_mode×opcode组合均正确执行返回STS_OK(0x00)；
+2.各lane_mode下接收拍数符合bpc计算：1-bit=48/1=48拍, 4-bit=48/4=12拍, 8-bit=48/8=6拍, 16-bit=48/16=3拍；
+3.Burst命令hburst映射正确：1→SINGLE, 4→INCR4, 8→INCR8, 16→INCR16；
+4.事务间pcs_n_i=1期间lane_mode切换正确生效；
 coverage check点：
-1.覆盖wdata[31:0]全0/全1/0xAAAAAAAA/随机值；
-2.覆盖addr[31:0]对齐地址空间</t>
-        </is>
-      </c>
-      <c r="D32" s="13" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>TC_031</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_error_inject</t>
-        </is>
-      </c>
-      <c r="C33" s="21" t="inlineStr">
-        <is>
-          <t>随机错误注入测试：遍历各类错误条件。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
+1.lane_mode × opcode 交叉覆盖率100%；
+2.burst_len × lane_mode 交叉覆盖率100%；
+3.所有FSM状态跳转至少被触发一次</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>TC_049</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>test_rand_ahb_single</t>
+        </is>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，随机lane_mode_i；
+2.AHB slave随机响应（大部分hready_i=1, hresp_i=0，偶尔hresp_i=1或延迟）；
 输入激励：
-1.随机选择错误类型并注入：
-   - 非法opcode(随机选择0x00~0x0F或0x24~0xFF)→验证STS_BAD_OPCODE(0x02)；
-   - 非法CSR地址(reg_addr随机&gt;=0x40)→验证STS_BAD_REG(0x10)；
-   - 非对齐地址(addr随机设置addr[1:0]!=2'b00)→验证STS_ALIGN_ERR(0x20)；
-   - 非法burst_len(随机选择2,3,5,6,7,9~15)→验证STS_BAD_BURST(0x80)；
-   - 跨1KB边界地址→验证STS_BURST_BOUND(0x81)；
-   - AHB错误响应(force hresp_i=1)→验证STS_AHB_ERR(0x40)；
-   - AHB超时(force hready_i=0持续256+周期)→验证STS_AHB_ERR(0x40)；
+1.随机选择AHB_WR32(opcode=0x20)或AHB_RD32(opcode=0x21)；
+2.随机生成4-byte对齐地址（addr[31:0]，addr[1:0]=2'b00）；
+3.对于写命令随机生成wdata(32-bit)；
+4.随机注入非对齐地址（addr[1:0]!=2'b00）验证ALIGN_ERR检测；
+5.重复执行N次（N≥200），混合正常和错误场景；
+期望结果：
+1.正常场景：STS_OK(0x00)，htrans_o序列NONSEQ→IDLE正确，hsize_o=3'b010；
+2.对齐错误：STS_ALIGN_ERR(0x20)，不发起AHB访问；
+3.hresp错误：STS_AHB_ERR(0x40)，axi_state经历AXI_ERR；
+4.AHB 2-phase流水时序正确：地址相与数据相错开1拍；
+coverage check点：
+1.覆盖opcode(AHB_WR32/AHB_RD32) × lane_mode所有组合；
+2.覆盖addr[1:0]所有4种取值；
+3.覆盖hresp_i=0/1场景</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>TC_050</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>test_rand_ahb_burst</t>
+        </is>
+      </c>
+      <c r="C52" s="21" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，随机lane_mode_i；
+2.AHB slave随机响应（大部分hready_i=1, hresp_i=0，偶尔延迟或错误）；
+输入激励：
+1.随机选择AHB_WR_BURST(0x22)或AHB_RD_BURST(0x23)；
+2.随机选择burst_len（遍历4/8/16）；
+3.随机生成4-byte对齐地址（确保不跨1KB边界：addr[9:0]+4·(burst_len-1)&lt;1024）；
+4.随机注入跨1KB边界地址验证BURST_BOUND检测；
+5.随机注入非法burst_len(2/3/5/6/7)验证BAD_BURST检测；n6.重复执行N次（N≥200），覆盖所有burst_len×读写组合；
+期望结果：
+1.正常Burst：STS_OK(0x00)，hburst_o映射正确，htrans: NONSEQ+SEQ×(N-1)；
+2.跨1KB边界：STS_BURST_BOUND(0x81)；
+3.非法burst_len：STS_BAD_BURST(0x80)；
+4.hburst_o在整个Burst期间保持稳定，haddr每拍+4；
+coverage check点：
+1.覆盖burst_len × opcode × lane_mode所有组合；
+2.覆盖hburst所有编码(SINGLE/INCR4/INCR8/INCR16)；
+3.覆盖1KB边界附近的地址场景</t>
+        </is>
+      </c>
+      <c r="D52" s="13" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>TC_051</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>test_rand_error_injection</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，随机lane_mode_i；
+2.随机选择测试场景（错误类型）；
+输入激励：
+1.随机选择错误类型并注入：非法opcode(0x00~0x0F或0x24~0xFF)、test_mode_i=0、en_i=0、非法CSR地址(reg_addr&gt;=0x40)、非对齐地址(addr[1:0]!=0)、非法burst_len(2,3,5,6,7,9~15)、跨1KB边界地址、AHB错误响应(force hresp_i=1)、AHB超时(force hready_i=0持续256+周期)、帧中途拉高pcs_n_i；
 2.每种错误类型重复执行N次（N≥10）；
+3.多错误同时注入验证优先级链：例如test_mode_i=0+en_i=0+bad_reg+align_err；
+4.每次错误后复位或等待事务结束再执行下一个；
 期望结果：
 1.前置错误：返回对应错误码，不发起CSR/AHB访问；
 2.AHB错误：返回STS_AHB_ERR(0x40)；
-3.错误后模块回到IDLE，可接受新命令；
-4.LAST_ERR寄存器保存最近错误码（sticky）；
+3.帧中止：返回STS_FRAME_ERR(0x01)（最高优先级）；
+4.多错误同时触发时仅返回最高优先级错误码；
+5.错误后模块可正常接受新命令；
 coverage check点：
 1.覆盖所有状态码：0x01, 0x02, 0x04, 0x08, 0x10, 0x20, 0x40, 0x80, 0x81；
-2.覆盖错误优先级链各组合</t>
-        </is>
-      </c>
-      <c r="D33" s="13" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>TC_032</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_lane_opcode_cross</t>
-        </is>
-      </c>
-      <c r="C34" s="21" t="inlineStr">
-        <is>
-          <t>交叉覆盖：所有lane_mode×所有opcode组合测试。
-配置条件：
+2.覆盖错误优先级链各组合；
+3.覆盖Burst中途错误中止场景</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>TC_052</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>test_rand_cross_lane_opcode</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
 1.模块复位完成，test_mode_i=1，en_i=1；
 2.使用嵌套循环遍历所有组合；
 输入激励：
-1.for lane_mode in [2'b00, 2'b01, 2'b10, 2'b11]：
-2.  配置lane_mode_i=lane_mode，等待2周期同步；
-3.  for opcode in [0x10, 0x11, 0x20, 0x21, 0x22, 0x23]：
-4.    发送对应opcode命令（合法参数）；
-5.    检查响应status_code=STS_OK(0x00)；
-6.    验证帧接收/发送拍数与lane_mode一致；
-期望结果：
-1.所有lane_mode×opcode组合均正常执行，返回STS_OK(0x00)；
-2.帧接收拍数=帧长/bpc，bpc=1/4/8/16对应各lane_mode；
-3.所有FSM状态跳转正确；
-4.lane_mode × opcode交叉覆盖率100%；
-coverage check点：
-1.lane_mode × opcode交叉覆盖率100%；
-2.所有FSM状态至少被触发一次</t>
-        </is>
-      </c>
-      <c r="D34" s="13" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>TC_033</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_burst_boundary</t>
-        </is>
-      </c>
-      <c r="C35" s="21" t="inlineStr">
-        <is>
-          <t>边界测试：最大burst_len、FIFO满/空边界、1KB地址边界。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送AHB_WR_BURST×16(opcode=0x22, burst_len=16, addr=0x10000000)，最大burst测试；
-2.发送AHB_RD_BURST×16(opcode=0x23, burst_len=16, addr=0x100003C0)，地址接近1KB边界但不跨越；
-3.发送AHB_RD_BURST×4(opcode=0x23, burst_len=4, addr=0x100003F0)，恰好在1KB边界内(addr+4*3=0x100003FC&lt;0x10000400)；
-4.发送AHB_RD_BURST×4(opcode=0x23, burst_len=4, addr=0x100003FC)，跨越1KB边界(addr+4*3=0x10000408&gt;=0x10000400)；
-5.发送burst_len=1的Burst命令验证退化为SINGLE；
-6.测试FIFO深度边界：连续执行burst_len=16命令使rxfifo_cnt接近32；
-期望结果：
-1.burst_len=16正常执行，hburst_o=INCR16(3'b111)；
-2.1KB边界内地址正常执行，返回STS_OK(0x00)；
-3.跨1KB边界返回STS_BURST_BOUND(0x81)；
-4.burst_len=1退化为SINGLE，hburst_o=SINGLE(3'b000)；
-5.FIFO满/空边界行为正确；
-coverage check点：
-1.覆盖burst_len边界值：1, 4, 8, 16；
-2.覆盖1KB地址边界场景(跨越/不跨越)；
-3.覆盖FIFO深度边界值</t>
-        </is>
-      </c>
-      <c r="D35" s="13" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>TC_034</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_csr_all_addr</t>
-        </is>
-      </c>
-      <c r="C36" s="21" t="inlineStr">
-        <is>
-          <t>随机CSR地址遍历：覆盖合法/非法/预留地址。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.遍历reg_addr=0x00(VERSION)~0x10(BURST_CNT)，每个执行RD_CSR(opcode=0x11)，记录返回状态码和rdata；
-2.遍历reg_addr=0x11~0x3F（预留/未实现），每个执行RD_CSR；
-3.随机选择reg_addr&gt;=0x40的非法地址（如0x40,0x7F,0xFF），执行RD_CSR和WR_CSR；
-4.重复执行N次（N≥50），每次随机选择地址；
-期望结果：
-1.reg_addr 0x00~0x10返回STS_OK(0x00)，csr_rd_en_o产生单周期脉冲；
-2.reg_addr&gt;=0x40返回STS_BAD_REG(0x10)，无csr_rd_en_o脉冲；
-3.RO寄存器写操作返回STS_OK但值不变；
-4.所有CSR访问时序正确（写1周期，读1周期延迟）；
-coverage check点：
-1.覆盖CSR地址空间0x00~0xFF；
-2.覆盖合法/非法/预留地址边界</t>
-        </is>
-      </c>
-      <c r="D36" s="13" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>TC_035</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_burst_len_sweep</t>
-        </is>
-      </c>
-      <c r="C37" s="21" t="inlineStr">
-        <is>
-          <t>随机burst_len遍历：合法值和非法值全覆盖。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.遍历合法burst_len={1,4,8,16}，发送AHB_RD_BURST命令(opcode=0x23)，验证hburst_o映射正确；
-2.遍历非法burst_len={2,3,5,6,7,9,10,11,12,13,14,15,17,31}，发送AHB_RD_BURST命令，验证返回STS_BAD_BURST(0x80)；
-3.随机选择burst_len值(0~31)，发送Burst命令，重复N次（N≥50）；
-4.验证burst_len=1时退化为SINGLE，hburst_o=SINGLE(3'b000)；
-期望结果：
-1.合法burst_len正确映射：1→SINGLE, 4→INCR4, 8→INCR8, 16→INCR16；
-2.非法burst_len返回STS_BAD_BURST(0x80)，不发起AHB访问；
-3.burst_len=0返回STS_BAD_BURST(0x80)；
-4.所有合法Burst正常完成，status_code=STS_OK(0x00)；
-coverage check点：
-1.覆盖burst_len全空间0~31；
-2.覆盖hburst_o所有编码：3'b000, 3'b011, 3'b101, 3'b111</t>
-        </is>
-      </c>
-      <c r="D37" s="13" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>TC_036</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_multi_cmd_sequence</t>
-        </is>
-      </c>
-      <c r="C38" s="21" t="inlineStr">
-        <is>
-          <t>随机多命令序列测试：混合不同opcode连续发送。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.随机生成命令序列（长度10~50条），每条随机选择opcode∈{0x10,0x11,0x20,0x21,0x22,0x23}；
-2.对每条命令使用随机合法参数（对齐地址、合法burst_len等）；
-3.连续发送命令，每条命令结束后（pcs_n_i=1→0）发送下一条；
-4.验证每条命令的status_code和响应数据；
-5.重复执行N次（N≥500次总命令），覆盖各种opcode排列组合；
-期望结果：
-1.所有命令正常完成，返回STS_OK(0x00)；
-2.每条命令执行后模块回到IDLE，可立即接受下一条命令；
-3.CSR/AHB接口时序正确：csr_wr_en_o/csr_rd_en_o单周期，htrans_o=NONSEQ/SEQ正确；
-4.Burst命令后FIFO清空，不影响后续命令；
-coverage check点：
-1.覆盖所有opcode连续执行序列；
-2.覆盖所有FSM状态跳转至少一次</t>
-        </is>
-      </c>
-      <c r="D38" s="13" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>TC_037</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_ahb_wait_states</t>
-        </is>
-      </c>
-      <c r="C39" s="21" t="inlineStr">
-        <is>
-          <t>随机AHB等待状态测试：验证hready_i随机等待下的正确性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.随机选择命令类型（AHB_WR32/AHB_RD32/AHB_WR_BURST/AHB_RD_BURST）；
-2.发送命令后，对每个AHB beat随机插入0~10周期hready_i=0等待；
-3.验证模块在等待期间axi_state=AXI_WAIT，timeout_cnt递增但不超过255；
-4.验证hready_i=1后数据正确采样/驱动；
-5.重复执行N次（N≥100），每次随机等待周期数；
-期望结果：
-1.所有命令正常完成，返回STS_OK(0x00)；
-2.等待期间htrans_o=IDLE，haddr_o保持；
-3.等待不超过255周期时不触发超时；
-4.Burst中每beat独立等待，数据正确；
-coverage check点：
-1.覆盖hready_i等待周期数0~10；
-2.覆盖AXI_WAIT状态持续时间</t>
-        </is>
-      </c>
-      <c r="D39" s="13" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>TC_038</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_burst_mid_error</t>
-        </is>
-      </c>
-      <c r="C40" s="21" t="inlineStr">
-        <is>
-          <t>随机Burst中途错误注入：INCR4/8/16中随机beat注入hresp_i=1。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送AHB_RD_BURST×8命令(opcode=0x23, burst_len=8, addr=0x10000000)；
-2.在随机beat(第1~7拍)注入hresp_i=1（错误响应）；
-3.观察axi_state跳转AXI_ERR，剩余beat取消；
-4.验证TXFIFO中已缓冲部分beat仍发往前端；
-5.分别测试INCR4(beat2注入)、INCR8(beat4注入)、INCR16(beat8注入)场景；
-6.每种场景重复N次（N≥10），随机选择出错beat位置；
-期望结果：
-1.hresp_i=1后axi_state跳转AXI_ERR，返回STS_AHB_ERR(0x40)；
-2.出错beat之后的beat不再发起（htrans_o=IDLE）；
-3.已缓冲beat正常发出；
-4.错误后模块自动恢复AXI_IDLE，可接受新命令；
-coverage check点：
-1.覆盖Burst出错beat位置1~burst_len-1；
-2.覆盖AXI_ERR状态跳转</t>
-        </is>
-      </c>
-      <c r="D40" s="13" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>TC_039</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_align_err</t>
-        </is>
-      </c>
-      <c r="C41" s="21" t="inlineStr">
-        <is>
-          <t>随机对齐错误测试：遍历所有非对齐地址组合。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送AHB_WR32命令(opcode=0x20)，addr[1:0]=2'b01（非4-byte对齐）；
-2.发送AHB_RD32命令(opcode=0x21)，addr[1:0]=2'b10；
-3.发送AHB_WR_BURST命令(opcode=0x22)，addr[1:0]=2'b11；
-4.随机选择非对齐地址(addr[1:0]∈{2'b01,2'b10,2'b11})，随机选择opcode∈{0x20,0x21,0x22,0x23}，重复N次（N≥30）；
-5.验证所有非对齐地址均返回STS_ALIGN_ERR(0x20)，不发起AHB访问；
-期望结果：
-1.所有addr[1:0]!=2'b00的AHB命令返回STS_ALIGN_ERR(0x20)；
-2.不产生htrans_o脉冲，AHB保持IDLE；
-3.CSR命令不受addr对齐约束（使用reg_addr而非addr）；
-4.错误后模块回到IDLE，可接受新命令；
-coverage check点：
-1.覆盖addr[1:0]所有非对齐取值：2'b01, 2'b10, 2'b11；
-2.覆盖STS_ALIGN_ERR与所有AHB opcode组合</t>
-        </is>
-      </c>
-      <c r="D41" s="13" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>TC_040</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_frame_abort_timing</t>
-        </is>
-      </c>
-      <c r="C42" s="21" t="inlineStr">
-        <is>
-          <t>随机帧中止时机测试：在帧接收各阶段随机提前拉高pcs_n_i。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送WR_CSR帧(48-bit)，在接收4bit后(opcode未锁存，&lt;8bit)提前拉高pcs_n_i；
-2.发送WR_CSR帧(48-bit)，在接收8bit后(opcode刚锁存)提前拉高pcs_n_i；
-3.发送WR_CSR帧(48-bit)，在接收24bit后(opcode已锁存但帧未完成)提前拉高pcs_n_i；
-4.随机选择提前拉高时机(rx_count: 4~47 bit随机)，重复N次（N≥30）；
-5.验证每种时机的返回状态码；
-期望结果：
-1.rx_count&lt;8(opcode未锁存)：静默复位，不产生frame_abort，不返回状态码；
-2.rx_count&gt;=8(opcode已锁存)：产生frame_abort，返回STS_FRAME_ERR(0x01)；
-3.所有帧中止场景不发起CSR/AHB访问；
-4.帧中止后模块回到IDLE，RXFIFO drain至empty；
-coverage check点：
-1.覆盖frame_abort触发时机(已锁存/未锁存)；
-2.覆盖rx_count从0到expected_rx_bits的各阶段</t>
-        </is>
-      </c>
-      <c r="D42" s="13" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>TC_041</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_timeout_threshold</t>
-        </is>
-      </c>
-      <c r="C43" s="21" t="inlineStr">
-        <is>
-          <t>超时阈值边界测试：验证BUS_TIMEOUT_CYCLES=256的精确边界。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送AHB_RD32命令，force hready_i=0持续254周期后释放→不应超时；
-2.发送AHB_RD32命令，force hready_i=0持续255周期后释放→达到阈值边界；
-3.发送AHB_RD32命令，force hready_i=0持续256周期→应触发超时；
-4.验证timeout_cnt==BUS_TIMEOUT_CYCLES-1(255)时AXI_ERR跳转；
-5.每种边界重复N次（N≥5）确认稳定性；
-期望结果：
-1.254周期等待不超时，hready_i=1后正常完成，返回STS_OK(0x00)；
-2.255周期等待不超时（计数值0~254共255个AXI_WAIT拍，未达255）；
-3.256周期等待触发超时，timeout_cnt达到255，axi_state→AXI_ERR，返回STS_AHB_ERR(0x40)；
-4.超时后自动恢复AXI_IDLE，可接受新命令；
-coverage check点：
-1.覆盖timeout_cnt边界值254,255,256；
-2.覆盖AXI_ERR跳转条件</t>
-        </is>
-      </c>
-      <c r="D43" s="13" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>TC_042</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_status_accumulation</t>
-        </is>
-      </c>
-      <c r="C44" s="21" t="inlineStr">
-        <is>
-          <t>随机状态累积测试：混合正常/错误命令，验证STATUS/LAST_ERR sticky行为。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.执行正常WR_CSR命令后读取STATUS(reg_addr=0x08)和LAST_ERR(reg_addr=0x0C)；
-2.执行错误命令(非对齐地址)后读取STATUS和LAST_ERR，验证CMD_ERR=1(sticky)，LAST_ERR=0x20；
-3.插入一条正常命令后再次读取LAST_ERR，验证sticky——错误码0x20仍存在；
-4.执行另一种错误(非法opcode)，验证LAST_ERR更新为新错误码0x02；
-5.重复混合正常/错误命令序列N次（N≥30），验证STATUS各bit和LAST_ERR更新规则；
-期望结果：
-1.正常命令后STATUS.BUSY=0, RESP_VALID=1；
-2.错误命令后对应STATUS sticky位=1，LAST_ERR保存错误码；
-3.中间插入正常命令不影响LAST_ERR（sticky保持）；
-4.新错误覆盖LAST_ERR为最新错误码；
-coverage check点：
-1.覆盖STATUS各bit位(BUSY,RESP_VALID,CMD_ERR,BUS_ERR,FRAME_ERR,IN_TEST_MODE,OUT_EN,BURST_ERR)；
-2.覆盖LAST_ERR各错误码的sticky更新行为</t>
-        </is>
-      </c>
-      <c r="D44" s="13" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>TC_043</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_dfx_counter</t>
-        </is>
-      </c>
-      <c r="C45" s="21" t="inlineStr">
-        <is>
-          <t>随机DFX计数器测试：验证统计计数器累加正确性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.依次执行6种opcode命令各K次（K≥5），验证每opcode成功计数器递增K；
-2.依次触发各类错误各M次（M≥3），验证每错误码失败计数器递增M；
-3.执行CSR读/写命令各P次（P≥5），验证CSR读/写计数器递增P；
-4.执行AHB Single读/写各Q次（Q≥5），验证AHB Single计数器递增Q；
-5.执行Burst命令(INCR4/8/16读/写)，验证Burst计数器和total_burst_beat_cnt；
-6.随机混合执行各类命令N次（N≥100），验证计数器累加正确；
-期望结果：
-1.每opcode成功计数=该opcode成功执行次数；
-2.每错误码失败计数=该错误码出现次数；
-3.total_burst_beat_cnt=Burst总beat数；
-4.写1清零(WC)后计数器归零；
-coverage check点：
-1.覆盖6路opcode成功计数 + 8路错误码计数；
-2.覆盖CSR/AHB/Burst各类计数器</t>
-        </is>
-      </c>
-      <c r="D45" s="13" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>TC_044</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_burst_1kb_boundary</t>
-        </is>
-      </c>
-      <c r="C46" s="21" t="inlineStr">
-        <is>
-          <t>随机1KB边界测试：精确验证跨1KB边界的地址判定。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送AHB_RD_BURST×4(opcode=0x23, burst_len=4, addr=0x100003F0)：addr[9:0]=0x3F0, addr+4*3=0x3FC&lt;0x400→不跨1KB；
-2.发送AHB_RD_BURST×4(opcode=0x23, burst_len=4, addr=0x100003FC)：addr[9:0]=0x3FC, addr+4*3=0x408&gt;=0x400→跨1KB；
-3.发送AHB_RD_BURST×16(opcode=0x23, burst_len=16, addr=0x100003C0)：addr+4*15=0x3FC→刚好不跨；
-4.随机生成跨越/不跨越1KB边界的地址，发送Burst命令，重复N次（N≥30）；
-期望结果：
-1.不跨1KB边界：正常执行，返回STS_OK(0x00)；
-2.跨1KB边界：返回STS_BURST_BOUND(0x81)，不发起AHB访问；
-3.判定公式：addr[9:0]+4·(burst_len-1)&gt;=1024；
-4.错误后模块回到IDLE，可接受新命令；
-coverage check点：
-1.覆盖1KB边界两侧地址；
-2.覆盖STS_BURST_BOUND(0x81)触发条件</t>
-        </is>
-      </c>
-      <c r="D46" s="13" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>TC_045</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_fifo_pressure</t>
-        </is>
-      </c>
-      <c r="C47" s="21" t="inlineStr">
-        <is>
-          <t>随机FIFO压力测试：反复产生RXFIFO/TXFIFO满/空场景。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.连续执行AHB_WR_BURST×16命令(opcode=0x22)，使RXFIFO反复达到满/非满状态；
-2.连续执行AHB_RD_BURST×16命令(opcode=0x23)，使TXFIFO反复达到空/非空状态；
-3.随机控制后端消费速率（插入0~5周期hready_i=0等待），产生不同FIFO占用水平；
-4.验证rxfifo_full_o/txfifo_empty_o状态信号与rxfifo_cnt/txfifo_cnt一致；
-5.重复执行N次（N≥20次Burst事务）；
-期望结果：
-1.RXFIFO满时rxfifo_full_o=1，接收暂停；非满时恢复接收；
-2.TXFIFO空时txfifo_empty_o=1，TX暂停但pdo_oe_o保持高；
-3.rxfifo_backpressure_cnt和txfifo_stall_cnt正确累加；
-4.所有Burst事务最终正确完成，数据无丢失；
-coverage check点：
-1.覆盖rxfifo_cnt/txfifo_cnt全范围(0~32)；
-2.覆盖rxfifo_full_o/txfifo_empty_o跳变</t>
-        </is>
-      </c>
-      <c r="D47" s="13" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>TC_046</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_lane_switch_legal</t>
-        </is>
-      </c>
-      <c r="C48" s="21" t="inlineStr">
-        <is>
-          <t>随机合法lane切换测试：仅在pcs_n_i=1时切换lane_mode_i。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.初始lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.在16-bit模式下执行WR_CSR命令；
-2.命令结束后(pcs_n_i=1)，随机选择新lane_mode_i∈{2'b00,2'b01,2'b10,2'b11}；
-3.等待2个clk_i周期同步后发送命令验证新模式工作正常；
-4.重复切换+执行N次（N≥50），每次随机选择lane_mode和命令类型；
-5.验证每次切换后命令按新lane_mode正确执行；
-期望结果：
-1.每次lane_mode切换后命令正常执行，返回STS_OK(0x00)；
-2.帧接收/发送拍数与新lane_mode的bpc一致；
-3.所有4种lane_mode均被遍历；
-4.切换过程中无数据损坏或FSM异常；
-coverage check点：
-1.覆盖lane_mode所有切换组合(4×4=16种)；
-2.覆盖每种lane_mode下的命令执行</t>
-        </is>
-      </c>
-      <c r="D48" s="13" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>TC_047</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_opcode_status_cross</t>
-        </is>
-      </c>
-      <c r="C49" s="21" t="inlineStr">
-        <is>
-          <t>操作码×状态码交叉覆盖测试。
-配置条件：
-1.模块复位完成；
-2.使用嵌套循环遍历所有opcode×成功/错误场景组合；
-输入激励：
-1.for opcode in [0x10, 0x11, 0x20, 0x21, 0x22, 0x23]：
-2.  for scenario in [success, frame_err, bad_opcode, not_in_test, disabled, bad_reg, align_err, ahb_err, bad_burst, burst_bound]：
-3.    配置对应条件（如test_mode_i=0触发not_in_test，非对齐地址触发align_err等）；
-4.    发送命令并检查status_code；
+1.for lane_mode in [2'b00, 2'b01, 2'b10, 2'b11]: for opcode in [0x10, 0x11, 0x20, 0x21, 0x22, 0x23]: for burst_len in [1, 4, 8, 16]（仅Burst命令）: for success_or_error in [success, error]: 配置对应条件，发送命令，检查响应；
+2.成功场景：合法参数配置；
+3.错误场景：随机注入1种错误条件（bad_opcode/not_in_test/disabled/bad_reg/align_err/bad_burst/burst_bound）；
+4.每个组合重复2次以上；
 期望结果：
 1.成功路径：status=STS_OK(0x00)；
-2.错误路径：返回正确错误码，符合优先级链；
-3.所有opcode×status_code组合被验证；
-4.CSR类opcode不产生ALIGN_ERR/BAD_BURST/BURST_BOUND（仅AHB类命令触发）；
-coverage check点：
-1.opcode × status_code交叉覆盖率100%；
-2.错误优先级链验证</t>
-        </is>
-      </c>
-      <c r="D49" s="13" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>TC_048</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_ahb_err_recovery</t>
-        </is>
-      </c>
-      <c r="C50" s="21" t="inlineStr">
-        <is>
-          <t>随机AHB错误恢复测试：注入错误后验证模块自动恢复并正常工作。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.发送AHB_RD32命令，force hresp_i=1触发STS_AHB_ERR(0x40)；
-2.验证模块回到IDLE后发送正常AHB_WR32命令(opcode=0x20, addr=0x10000000, wdata=0x12345678)；
-3.发送AHB_RD_BURST×4命令，在第2 beat注入hresp_i=1；
-4.验证Burst中止后发送正常Burst命令；
-5.重复错误→恢复序列N次（N≥20），每次随机选择错误类型和恢复命令；
-期望结果：
-1.Single AHB错误后：axi_state→AXI_ERR→AXI_IDLE，新命令正常执行；
-2.Burst中途错误后：剩余beat取消，TXFIFO drain，新命令正常执行；
-3.AHB输出恢复空闲：htrans_o=IDLE, hburst_o=SINGLE, haddr_o=0；
-4.RX/TX FIFO在错误后drain至empty；
-coverage check点：
-1.覆盖AXI_ERR→AXI_IDLE恢复路径；
-2.覆盖Single/Burst错误后恢复</t>
-        </is>
-      </c>
-      <c r="D50" s="13" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>TC_049</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_burst_wr_readback</t>
-        </is>
-      </c>
-      <c r="C51" s="21" t="inlineStr">
-        <is>
-          <t>随机Burst写后读回验证：验证数据一致性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.随机选择burst_len∈{4,8,16}和地址addr(4-byte对齐，不跨1KB边界)；
-2.发送AHB_WR_BURST命令(opcode=0x22)，写入N个随机32-bit数据；
-3.发送AHB_RD_BURST命令(opcode=0x23)，从同一地址读回N个数据；
-4.逐beat比较写入数据和读回数据是否一致；
-5.重复执行N次（N≥30），每次随机burst_len、地址和数据；
-期望结果：
-1.写命令返回STS_OK(0x00)；
-2.读命令返回STS_OK(0x00) + N beat rdata；
-3.每个beat读回数据=写入数据，数据一致性100%；
-4.hburst_o映射正确：burst_len→INCR4/8/16；
-coverage check点：
-1.覆盖burst_len={4,8,16} × 读/写组合；
-2.覆盖数据一致性验证</t>
-        </is>
-      </c>
-      <c r="D51" s="13" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>TC_050</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_csr_attr_verify</t>
-        </is>
-      </c>
-      <c r="C52" s="21" t="inlineStr">
-        <is>
-          <t>随机寄存器属性验证：对每个CSR执行写-读序列验证RO/RW/WC属性。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.VERSION(0x00)RO验证：RD_CSR读复位值→WR_CSR写0xFFFFFFFF→RD_CSR读回验证值不变→证明RO属性；
-2.CTRL(0x04)RW验证：WR_CSR写0x0000000F(EN=1,LANE_MODE=11,SOFT_RST=1)→RD_CSR读回0x0000000F→证明RW属性；
-3.STATUS(0x08)RO验证：RD_CSR读当前值→WR_CSR写0xFF→RD_CSR读回验证硬件值而非0xFF→证明RO属性；
-4.LAST_ERR(0x0C)RO验证：触发错误后RD_CSR读LAST_ERR→WR_CSR写0x00→RD_CSR读回验证错误码不变→证明RO属性(sticky)；
-5.BURST_CNT(0x10)WC验证：执行Burst后RD_CSR读非零值→WR_CSR写0x00000001→RD_CSR读回0x0000→证明WC属性(写1清零)；
-6.重复对每个寄存器执行写-读序列N次（N≥5），确保属性验证充分；
-期望结果：
-1.RO寄存器(VERSION/STATUS/LAST_ERR)：写操作不影响值，读回写入前值；
-2.RW寄存器(CTRL)：写入后读回一致；
-3.WC寄存器(BURST_CNT)：写1清零，写非1不清零或按实现定义；
-4.所有CSR访问时序正确；
-coverage check点：
-1.覆盖所有5个CSR寄存器的属性验证(RO/RW/WC)；
-2.覆盖写-读回序列</t>
-        </is>
-      </c>
-      <c r="D52" s="13" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>TC_051</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_priority_chain</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>随机优先级链验证：单独测试每个错误条件，再测试组合，证明优先级。
-配置条件：
-1.模块复位完成，lane_mode_i=2'b11(16-bit模式)；
-输入激励：
-1.单独测试STS_FRAME_ERR：发送命令中途拉高pcs_n_i→验证返回0x01；
-2.单独测试STS_BAD_OPCODE：发送opcode=0xFF→验证返回0x02；
-3.单独测试STS_NOT_IN_TEST：设置test_mode_i=0→发送命令→验证返回0x04；
-4.单独测试STS_DISABLED：设置en_i=0→发送命令→验证返回0x08；
-5.单独测试STS_BAD_REG：发送reg_addr=0x40→验证返回0x10；
-6.单独测试STS_ALIGN_ERR：发送addr[1:0]!=0→验证返回0x20；
-7.组合测试：设置test_mode_i=0且en_i=0且发送非法opcode→验证返回最高优先级STS_FRAME_ERR或STS_BAD_OPCODE（取决于帧是否完整接收）；
-8.组合测试：发送Burst命令(burst_len=5非法)+非对齐地址→验证STS_ALIGN_ERR(0x20)&gt;STS_BAD_BURST(0x80)；
-期望结果：
-1.单独条件：返回对应错误码，与LRS一致；
-2.组合条件：返回优先级链中最高优先级错误码；
-3.优先级链(高→低)：FRAME_ERR(0x01)&gt;BAD_OPCODE(0x02)&gt;NOT_IN_TEST(0x04)&gt;DISABLED(0x08)&gt;BAD_REG(0x10)&gt;ALIGN_ERR(0x20)&gt;BAD_BURST(0x80)&gt;BURST_BOUND(0x81)；
-4.STS_AHB_ERR(0x40)与前置错误互斥；
-coverage check点：
-1.覆盖优先级链所有8级错误码；
-2.覆盖多错误条件组合场景</t>
-        </is>
-      </c>
-      <c r="D53" s="13" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>TC_052</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_performance_measurement</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>随机性能测量：各lane_mode×burst_len组合，测量有效吞吐。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.AHB zero-wait-state环境；
-输入激励：
-1.for lane_mode in [2'b00, 2'b01, 2'b10, 2'b11]：
-2.  配置lane_mode_i，等待2周期同步；
-3.  发送AHB_WR_BURST×16命令，测量端到端延时(从pcs_n_i拉低到拉高的总周期数)；
-4.  发送AHB_RD_BURST×16命令，测量端到端延时；
-5.  计算有效吞吐=64B/总周期数×clk_i频率；
-期望结果：
-1.16-bit lane下AHB_WR_BURST×16有效吞吐约116MB/s；
-2.16-bit lane下AHB_RD_BURST×16有效吞吐约118MB/s；
-3.各lane_mode吞吐比例与线速比例一致(1:4:8:16)；
-4.1-bit lane下约7.5MB/s，4-bit约30MB/s，8-bit约60MB/s；
-coverage check点：
-1.覆盖4种lane_mode × 2种Burst方向(读/写)；
-2.覆盖有效吞吐量化验证</t>
-        </is>
-      </c>
-      <c r="D54" s="13" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>TC_053</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>test_rand_cg_full_cross</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>全交叉覆盖测试：lane_mode×opcode×burst_len×success|error完整交叉。
-配置条件：
-1.模块复位完成；
-2.使用嵌套循环遍历所有组合；
-输入激励：
-1.for lane_mode in [2'b00, 2'b01, 2'b10, 2'b11]：
-2.  for opcode in [0x10, 0x11, 0x20, 0x21, 0x22, 0x23]：
-3.    for burst_len in [1, 4, 8, 16]：  // 仅Burst命令
-4.      for success_or_error in [success, error]：
-5.        配置对应条件，发送命令，检查响应；
-6.        成功场景：合法参数，验证STS_OK；
-7.        失败场景：注入对应错误，验证正确错误码；
-期望结果：
-1.成功路径：status=STS_OK(0x00)；
-2.失败路径：返回正确错误码，符合优先级链；
-3.所有组合均被验证；
-4.功能覆盖率100%；
+2.失败路径：返回正确错误码，优先级链正确；
+3.所有lane_mode×opcode组合均被验证；
+4.所有FSM状态跳转至少被触发一次；
 coverage check点：
 1.lane_mode × opcode × (success|error) 交叉覆盖率100%；
 2.burst_len × lane_mode 交叉覆盖率100%；
 3.所有FSM状态跳转至少被触发一次</t>
         </is>
       </c>
+      <c r="D54" s="13" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>TC_053</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>test_rand_fifo_pressure</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
+2.AHB slave随机延迟响应（hready_i随机0~3周期等待）；
+输入激励：
+1.连续发送AHB_WR_BURST×16命令，制造RXFIFO满反压场景；
+2.连续发送AHB_RD_BURST×16命令，制造TXFIFO空等待场景；
+3.随机混合Burst读写命令，验证FIFO在不同压力下的行为；
+4.每个Burst事务间等待pcs_n_i=1至少2周期；
+5.重复执行N次（N≥50）；
+期望结果：
+1.RXFIFO满时：rxfifo_full_o=1, rx_shift_en暂停，后端消费后恢复；
+2.TXFIFO空时：txfifo_empty_o=1, pdo_oe_o保持高, pdo_o保持上一拍数据；
+3.FIFO深度32足够覆盖burst_len=16场景；
+4.反压期间数据不丢失，最终全部正确传输；
+5.所有命令返回STS_OK(0x00)；
+coverage check点：
+1.覆盖RXFIFO/TXFIFO在各种压力下的行为；
+2.覆盖rxfifo_full和txfifo_empty场景</t>
+        </is>
+      </c>
       <c r="D55" s="13" t="n"/>
     </row>
     <row r="56">
@@ -5889,29 +5986,30 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>test_rand_backpressure_stress</t>
+          <t>test_rand_burst_len_boundary</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>反压压力测试：持续运行Burst事务，反复产生FIFO满/空场景。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，随机lane_mode_i；
+2.AHB slave正常响应；
 输入激励：
-1.连续执行100次AHB_WR_BURST×16命令(opcode=0x22)，随机插入后端等待(0~3周期hready_i=0)；
-2.连续执行100次AHB_RD_BURST×16命令(opcode=0x23)，随机插入后端等待；
-3.交替执行AHB_WR_BURST和AHB_RD_BURST，模拟实际工作负载；
-4.验证每次事务的status_code和rxfifo_cnt/txfifo_cnt状态；
-5.验证rxfifo_backpressure_cnt和txfifo_stall_cnt累加正确；
+1.随机选择burst_len（遍历1/4/8/16合法值和2/3/5/6/7/9~15非法值）；
+2.对于合法burst_len，随机选择1KB边界附近的地址（刚好不越界、刚好越界、越界1 beat）；
+3.对于非法burst_len，验证BAD_BURST(0x80)检测不受地址影响；
+4.随机选择WR_BURST/RD_BURST；
+5.重复执行N次（N≥100），覆盖所有burst_len×边界场景组合；
 期望结果：
-1.所有200+次Burst事务正确完成，无数据丢失；
-2.FIFO反压行为正确：满时暂停，空时等待；
-3.计数器正确累加，写1清零后归零；
-4.模块无死锁，连续运行稳定；
+1.合法burst_len+不越界地址：STS_OK(0x00)；
+2.合法burst_len+越界地址：STS_BURST_BOUND(0x81)；
+3.非法burst_len：STS_BAD_BURST(0x80)，不受地址影响；
+4.BAD_BURST(0x80)优先级高于BURST_BOUND(0x81)；
+5.所有前置错误均不发起AHB访问；
 coverage check点：
-1.覆盖RXFIFO/TXFIFO全范围占用水平；
-2.覆盖持续反压场景稳定性</t>
+1.覆盖burst_len所有合法和非法取值；
+2.覆盖1KB边界附近地址场景；
+3.覆盖BAD_BURST/BURST_BOUND错误码</t>
         </is>
       </c>
       <c r="D56" s="13" t="n"/>
@@ -5924,39 +6022,69 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>test_rand_fsm_state_coverage</t>
+          <t>test_csr_register_attr</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>FSM状态覆盖测试：设计激励确保所有FSM状态和状态跳转至少被触发一次。
-配置条件：
-1.模块复位完成，test_mode_i=1，en_i=1；
-2.lane_mode_i=2'b11(16-bit模式)；
+          <t>配置条件：
+1.模块复位完成，test_mode_i=1，en_i=1，lane_mode_i=2'b11(16-bit模式)；
 输入激励：
-1.触发front_state所有6态：IDLE(空闲)→ISSUE(发送WR_CSR)→WAIT_RESP→TA→TX→IDLE；再触发TX_BURST(发送AHB_RD_BURST)；
-2.触发back_state所有7态：S_IDLE→S_LOAD_TASK→S_EXEC(CSR路径)→S_BUILD_RESP→S_DONE；再走AHB Single→S_WAIT_AHB；再走Burst→S_BURST_LOOP；
-3.触发axi_state所有6态：AXI_IDLE→AXI_REQ→AXI_WAIT→AXI_DONE→AXI_IDLE；触发AXI_BURST(INCR4)；触发AXI_ERR(hresp_i=1)；
-4.触发所有front_state frame_abort跳转：ISSUE时abort→IDLE，WAIT_RESP时abort→IDLE；
-5.验证每个FSM状态跳转至少被触发1次；
+1.向VERSION(0x00, RO)写入0xDEADBEEF，再RD_CSR读回，验证写入无效（值不变）；
+2.向CTRL(0x04, RW)写入0x00000007(EN=1, LANE_MODE=2'b11, SOFT_RST=1)，RD_CSR读回验证0x00000007；
+3.向STATUS(0x08, RO)写入0xFFFFFFFF，RD_CSR读回验证写入无效（值不变）；
+4.向LAST_ERR(0x0C, RO)写入0x00000081，RD_CSR读回验证写入无效；
+5.向BURST_CNT(0x10, WC)写入0x00000001清零，再写入0x00000000验证写0不清零；
+6.对VERSION和STATUS分别做写入-回读对比，证明RO属性需先写再读确认值不变；
 期望结果：
-1.front_state: IDLE/ISSUE/WAIT_RESP/TA/TX/TX_BURST全部覆盖；
-2.back_state: S_IDLE/S_LOAD_TASK/S_EXEC/S_WAIT_AHB/S_BURST_LOOP/S_BUILD_RESP/S_DONE全部覆盖；
-3.axi_state: AXI_IDLE/AXI_REQ/AXI_BURST/AXI_WAIT/AXI_DONE/AXI_ERR全部覆盖；
-4.所有FSM状态跳转至少被触发1次；
+1.VERSION(RO)：写入后读回仍为复位默认值，证明RO——写入无效；
+2.CTRL(RW)：写入0x07后读回0x07，证明RW——写入值可读回；
+3.STATUS(RO)：写入后读回仍为硬件更新的当前值，证明RO——写入无效；
+4.LAST_ERR(RO)：写入后读回仍为sticky值，证明RO——写入无效；
+5.BURST_CNT(WC)：写1清零成功，写0不清零，证明WC属性；
 coverage check点：
-1.front_state_cp: coverpoint front_state {bins states[]={[0:5]}}；
-2.back_state_cp: coverpoint back_state {bins states[]={[0:6]}}；
-3.axi_state_cp: coverpoint axi_state {bins states[]={[0:5]}}；
-4.所有状态跳转至少被触发一次</t>
+对5个CSR寄存器的RO/RW/WC属性验证场景收集功能覆盖率</t>
         </is>
       </c>
       <c r="D57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
-      <c r="B58" s="2" t="n"/>
-      <c r="C58" s="3" t="n"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>TC_056</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>test_rand_full_scenario</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>配置条件：
+1.模块复位完成，随机配置test_mode_i和en_i；
+2.随机配置lane_mode_i；
+3.AHB slave随机响应（hready_i/hresp_i随机）；
+输入激励：
+1.随机选择opcode（遍历0x10~0x23+非法值0x00~0xFF）；
+2.随机选择burst_len（遍历1/4/8/16+非法值）；
+3.随机生成地址（对齐/非对齐/跨1KB边界随机混合）；
+4.随机生成wdata；
+5.随机注入错误条件（帧中止、AHB错误/超时）；
+6.重复执行N次（N≥500），覆盖所有合理配置和激励的组合；
+期望结果：
+1.成功路径：status=STS_OK(0x00)；
+2.失败路径：返回正确错误码，优先级链正确；
+3.所有前置错误均不发起CSR/AHB访问；
+4.AHB错误后模块可自动恢复至IDLE接受新命令；
+5.所有配置组合均被覆盖；
+coverage check点：
+1.覆盖lane_mode × opcode × (success|error) 交叉覆盖率100%；
+2.覆盖burst_len × lane_mode 交叉覆盖率100%；
+3.所有FSM状态跳转至少被触发一次；
+4.覆盖所有状态码</t>
+        </is>
+      </c>
       <c r="D58" s="4" t="n"/>
     </row>
     <row r="59">

</xml_diff>